<commit_message>
tracker QA: Sonnet completion pass, Opus adversarial referee (no invented content; boilerplate/positional/identical-cell defects), Sonnet fix pass, orchestrator re-check; rows 210-460 now stand alone with [ID n] cross-references; manifest Locke DOI corrected
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I460"/>
+  <dimension ref="A1:I461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9535,7 +9535,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Bogaert et al. 2022 (ABSTRACT) estimates *both* transition and emission parameters from real classified series and explicitly handles missing dates. *Inference:* the missing-data handling transfers directly to our irregular calendar; the estimation itself would be circular here, because eleven of our twelve years are 2020 projections (§2.3) — an EM fit would learn and reinforce the labeling error.</t>
+          <t>Bogaert et al. 2022 (ABSTRACT) estimates *both* transition and emission parameters from real classified series and explicitly handles missing dates. *Inference:* the missing-data handling transfers directly to the project's irregular calendar; the estimation itself would be circular here, because eleven of the project's twelve years are 2020 projections (§2.3) — an EM fit would learn and reinforce the labeling error.</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Filed under §2.3 — temporal chain, transitions, emissions. (full text, verified 2026-09-11; issue number corrected from 8(10)).</t>
+          <t>Miller et al. 2013 supplies the closest published analogue to the framework's persistence prior (framework §2.3): a multi-season occupancy model whose latent binary state carries both a non-detection rate and a false-positive rate in its emission, and estimates colonization/extinction transitions while correcting for both error rates.</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -9657,7 +9657,11 @@
           <t>Bayesian Modelling of Multi-Year Crop Type Classification Using Deep Neural Networks and Hidden Markov Models</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F214" t="inlineStr">
         <is>
           <t>Perantoni et al. 2025 (PRIMARY, arXiv HTML) reports F1 70.88 → 73.59 from adding an HMM layer, and states that evaluating on parcels that actually changed is future work.</t>
@@ -9746,7 +9750,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Filed under §2.3 — temporal chain, transitions, emissions; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought in round 1 for framework §2.3's persistence-prior literature on how transition probabilities are set in multi-temporal land-cover mapping; filed at METADATA grade with the contextual Markovian-kernel method named in its title, not yet read beyond the header.</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -9789,7 +9793,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Filed under §2.3 — temporal chain, transitions, emissions. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Yang et al. 2020 grades each pixel by the joint probability of its observed sequence under the HMM as a reliability score, rather than only emitting the Viterbi label — the cheapest companion instrument the review found for framework §2.3, obtainable from the forward-backward pass already computed.</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -9832,7 +9836,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Filed under §2.3 — temporal chain, transitions, emissions. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought in round 1 for framework §2.3's transition-estimation thread (continuous change detection and classification by HMM, applied to Beijing); filed, not yet read.</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -9875,7 +9879,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Benedek &amp; Sziranyi 2009 folds a spatial layer and a change layer into one joint mixed-Markov energy for bitemporal aerial imagery across large seasonal and sensor gaps — closer in spirit to this project's cross-flight problem than most Landsat-cadence work (framework §4.1).</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -9918,7 +9922,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Companion multilayer Markov random field paper to Benedek &amp; Sziranyi 2009 [ID 218, Benedek &amp; Sziranyi 2009], extending the joint spatial/change energy to a multilayer MRF for optical remote-sensing change detection (framework §4.1); filed, not yet read.</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -9961,7 +9965,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. (confirmed unreadable 2026-09-11: no OA/repository copy, five Sci-Hub mirrors empty).</t>
+          <t>Hoberg et al. 2015 is a pairwise CRF spanning multiple epochs and resolutions in one energy — structurally the closest architecture to what framework §4.1 wants; the 2015 IEEE TGRS journal version stays unreadable (no OA or repository copy found), so it is graded from its abstract and the read 2012 precursor [ID 221, Hoberg et al. 2012].</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -10004,7 +10008,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. (2012 precursor to the above; full text parsed 2026-09-11, §4.2).</t>
+          <t>Hoberg, Rottensteiner &amp; Heipke 2012 is the read precursor to Hoberg et al. 2015 [ID 220, Hoberg et al. 2015]: its pairwise CRF sets the spatial and temporal interaction weights beta and gamma 'empirically' with no value printed, confirming framework §4.1's 'no measured local/global weight' finding, and its transition table assigns 1.0 to class-preserving entries — a fourth documented instance of the laundering prior.</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -10047,7 +10051,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Liu, Song, Lu &amp; Xia 2021 stages spatial smoothing first, then an EM-trained HMM — negative evidence on ordering for framework §4.1: smoothing spatially before the temporal stage bakes spatial-consensus error into the sequence before the temporal chain ever sees a raw per-cell observation.</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -10090,7 +10094,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Filed under §4.1 — joint space and time. (full text via GFZ Potsdam repository mirror, verified 2026-09-11, §4.2).</t>
+          <t>Martinis &amp; Twele 2010 gates which units enter a spatio-temporal contextual update at all by an entropy-based confidence measure, admitting only nodes whose marginal-posterior entropy exceeds the scene's own mean — the nearest published mechanism to framework §4.1's graded local/global weight, though its own spatial and temporal weights are hand-fixed at 1 and never swept.</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -10133,7 +10137,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought in round 1 for framework §6.1's trajectory-segmentation family (a LandTrendr multispectral ensemble for forest disturbance detection); filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -10176,7 +10180,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Murakami &amp; Tsutsumida 2025 (METADATA): all three top out below 80% F1 (CCDC 78.14%) once the domain is urban rather than forest. *Inference:* the accuracy ceiling drops in exactly the direction we are moving.</t>
+          <t>Murakami &amp; Tsutsumida 2025 (METADATA): all three top out below 80% F1 (CCDC 78.14%) once the domain is urban rather than forest. *Inference:* the accuracy ceiling drops in exactly the direction this project is moving.</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -10219,7 +10223,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Pasquarella et al. 2022 confirms from primary text that both canonical trajectory segmenters — LandTrendr's regression vertices, CCDC's harmonic coefficients — replace every observation inside a stable segment with a fitted model value, placing trajectory segmentation at framework §6.1's 'apply the consensus shape' end of the spectrum rather than the conservative fill-or-veto end. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -10234,7 +10238,7 @@
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -10262,7 +10266,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Polunchenko &amp; Tartakovsky 2012 surveys sequential change-point detection for Bernoulli sequences with known pre- and post-change parameters — CUSUM, Shiryaev-Roberts, GLR — which is literally the arithmetic framework §2.3 needs; no remote-sensing paper applying this to a binary land-cover mask with pre-measured per-epoch recall and false-positive rates was found. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -10277,7 +10281,7 @@
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -10305,7 +10309,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Reiche, de Bruin, Hoekman, Verbesselt &amp; Herold 2015 holds a provisional change call pending and either confirms or drops it as later Landsat/ALOS PALSAR observations arrive — the closest published analog to framework §6.1's 'fill or veto single cells, never redraw' design.</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -10348,7 +10352,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Reiche et al. 2021 describes the operational RADD alert system for the Congo Basin (Sentinel-1), which reports user's accuracy 97.6% and producer's accuracy 95.0% for confirmed alerts &gt;=0.2 ha under the same confirm-or-reject dynamic as Reiche et al. 2015 [ID 228, Reiche et al. 2015], though its statistics assume 6-12 day revisit.</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -10391,7 +10395,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Rodman et al. 2021 (PRIMARY — full published PDF read 2026-09-11; bronze OA link dead, Unpaywall reports closed, retrieved via Sci-Hub mirror): detectability tracks disturbance severity and agent, confirmed with real numbers, not the qualitative paraphrase this entry previously carried. LandTrendr caught 74.3% of fire disturbances within one year vs. 26.5% of spruce-beetle mortality; even restricted to the 30.1% of beetle events with a confident onset year, detection was still 61.8% — 12.5 points below fire. The severity–detectability relationship is positive for *both* agents (β = 0.98, p &lt; 0.01). Net areal effect: LandTrendr mapped 37–41% less disturbed area than perimeter/index-based reference methods.</t>
+          <t>Rodman et al. 2021 (PRIMARY — full published PDF read 2026-09-11) confirms with real numbers that detectability tracks disturbance severity and agent: LandTrendr caught 74.3% of fire disturbances within one year vs. 26.5% of spruce-beetle mortality, and even restricted to confident-onset-year beetle events, detection was still 61.8% — 12.5 points below fire. The severity–detectability relationship is positive for both agents (β = 0.98, p &lt; 0.01). Net areal effect: LandTrendr mapped 37–41% less disturbed area than perimeter/index-based reference methods.</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -10434,7 +10438,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Verbesselt, Hyndman, Newnham &amp; Culvenor 2010 (BFAST) detects steps larger than 0.1 NDVI under stated noise but needs roughly 23 observations per year to identify a seasonal term; framework §6.1 notes this does not transfer to an archive with under one observation per year and no continuous index. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -10449,7 +10453,7 @@
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -10477,7 +10481,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought in round 1 for framework §6.1's trajectory-segmentation family (robust online Bayesian deforestation monitoring); filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -10520,7 +10524,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Filed under §6.1 — reshaping, segmentation, confirm-or-veto; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Zhu &amp; Woodcock 2014 (CCDC) requires three consecutive threshold-exceeding observations before flagging a break — a duration test rather than a prior-versus-evidence odds ratio — and reports producer's accuracy 98% / user's accuracy 86% for change; framework §2.3 shows this duration rule does not port to this project's measured miss rate. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -10535,7 +10539,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -10563,7 +10567,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Filed under §4.2 — ancillary and cadastral priors; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought in round 1 for framework §4.2's ancillary and cadastral priors (Bayesian updating of land-cover estimates in a data-rich environment); filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -10599,10 +10603,14 @@
           <t>City of Seattle Tree Canopy Assessment: Final Report (2016–2021)</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>N/A — agency report</t>
+        </is>
+      </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>City of Seattle 2023 (PRIMARY, 32-page PDF read incl. appendix tables) is the cleanest instance and the most locally relevant source in the review. Redevelopment parcels are 1.0% of city land but account for 13.7% of citywide net loss; by zone, 2.9% of Multifamily land carries 78% of that zone's net loss. *Inference, and it is load-bearing:* those are net-over-net ratios. Calibrating q_loss needs gross flip rates, which the report does not break out; the gross upper bound is ~4.9% citywide. Do not carry the 13.7–78% figures into a prior without that correction.</t>
+          <t>City of Seattle 2023 (PRIMARY, 32-page PDF read incl. appendix tables) is the cleanest instance and the most locally relevant source in the review: redevelopment parcels are 1.0% of city land but account for 13.7% of citywide net loss, and 2.9% of Multifamily land carries 78% of that zone's net loss. Inference, and it is load-bearing: those are net-over-net ratios, and calibrating q_loss needs gross flip rates, which the report does not break out (gross upper bound ~4.9% citywide). Do not carry the 13.7–78% figures into a prior without that correction. (Status corrected to To Read: no PDF on disk and review §8 lists it only as an agency report, no read route.)</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -10617,7 +10625,7 @@
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10696,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Pedley &amp; Morgenroth 2025 (Sustainable Cities and Society, PRIMARY — full publisher-paginated PDF via the UC repository, hdl 10092/108884, read 2026-09-11) is the fourth paper in this group, and its own numbers cut *against* a development-loss prior at the citywide scale even while confirming one at the parcel scale. Table 2: redeveloped properties are 2.33% of the 72,671 treed residential properties studied and carry only 12.78% of citywide canopy loss — 87.22% of all loss sits on unmodified land ("over 87% of the total loss occurred on unmodified properties with no recorded building work for new residential units").</t>
+          <t>Pedley &amp; Morgenroth 2025 (Sustainable Cities and Society, PRIMARY — full publisher-paginated PDF via the UC repository, hdl 10092/108884, read 2026-09-11) is one of four Christchurch-group papers on redevelopment-driven canopy loss (alongside Ossola &amp; Hopton 2017 [ID 236, Ossola &amp; Hopton 2017], Guo et al. 2018/2019 [ID 354-355], and Morgenroth et al. 2017 [ID 358, Morgenroth et al. 2017]), and its own numbers cut *against* a development-loss prior at the citywide scale even while confirming one at the parcel scale. Table 2: redeveloped properties are 2.33% of the 72,671 treed residential properties studied and carry only 12.78% of citywide canopy loss — 87.22% of all loss sits on unmodified land ("over 87% of the total loss occurred on unmodified properties with no recorded building work for new residential units").</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -10731,7 +10739,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Filed under §4.2 — ancillary and cadastral priors; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Rosa, Purves, Souza &amp; Ewers 2013 (PRIMARY, full text via PLOS ONE's open-access article page) is the sharpest warning in framework §4.2: an ancillary-layer-modulated deforestation prior reached AUC 0.92 and put roughly 80% of cumulative deforestation within 10 km of its predicted high-probability areas, while matching the predicted location and year exactly only about 2% of the time. This is a where-versus-when failure any development-prior validation must score by year, not only place.</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -10774,7 +10782,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. (author postprint via HAL, verified 2026-09-11).</t>
+          <t>Sought under framework §4.3 for cross-sensor domain-adaptation methods bearing on lidar-as-teacher transfer (multisensor temporal unsupervised domain adaptation for land cover mapping); full text obtained via HAL, not discussed further in the review's findings section.</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -10817,7 +10825,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought under framework §4.3 for lidar-as-teacher canopy-height mapping precedent (high-resolution multi-temporal forest canopy height mapping in California using GEDI lidar and multi-sensor remote sensing); filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -10853,10 +10861,14 @@
           <t>Super-Resolved Canopy Height Mapping from Sentinel-2 Time Series Using Airborne LiDAR HD</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. (preprint) Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under framework §4.3 for the lidar-as-teacher contract (super-resolved canopy-height mapping from Sentinel-2 time series using airborne lidar HD as the training target); an arXiv preprint, not yet read.</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -10892,10 +10904,14 @@
           <t>Forest canopy height estimation from satellite RGB imagery using large-scale airborne LiDAR-derived training data</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. (preprint).</t>
+          <t>Lai et al. 2026 estimates forest canopy height from satellite RGB imagery using large-scale airborne-lidar-derived training data — the same train-on-lidar, deploy-lidar-free contract framework §4.3 requires; an arXiv preprint, not yet read.</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -10981,7 +10997,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Lopez-Paz, Bottou, Schoelkopf &amp; Vapnik 2016 defines privileged information as present at training and structurally absent at inference, with generalized distillation as the teacher/student form — the contract framework §4.3's lidar-as-teacher design must satisfy.</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -11017,10 +11033,14 @@
           <t>Capturing Temporal Dynamics in Large-Scale Canopy Tree Height Estimation</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. (preprint) Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Pauls et al. 2025 addresses temporal dynamics in large-scale canopy tree-height estimation under the same lidar-as-teacher framing as framework §4.3; an arXiv preprint, not yet read.</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -11149,7 +11169,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Vapnik &amp; Vashist 2009 is the origin statement that privileged information is present at training and structurally absent at inference — the definition Lopez-Paz et al. 2016 [ID 244, Lopez-Paz et al. 2016] formalises as generalized distillation for framework §4.3.</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -11192,7 +11212,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Filed under §4.3 — privileged information, lidar as teacher, cross-year transfer. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under framework §4.3 for training-data selection practice in an operational annual land-cover product (LCMAP); filed, not obtained.</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -11235,7 +11255,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution; grade ABSTRACT, no further reviewer note recorded in the bibliography.</t>
+          <t>Brown et al. 2022 held ground sample distance fixed at 0.5 m/px and varied only the optical point-spread function, moving detector mAP by more than 50% from aperture type alone — outside confirmation, in animal detection rather than canopy mapping, that season and sensor can dominate over nominal resolution (framework §4.4).</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -11278,7 +11298,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought under framework §4.4 for a label-taxonomy curriculum precedent (coarse-to-fine semantic segmentation of satellite images); filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -11321,7 +11341,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under framework §4.4 for deep-supervision architectures on aerial imagery (multi-scale shuffling CNNs with deep supervision, ISPRS Annals); filed in the acquisition pass, not yet read.</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -11364,7 +11384,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Lee, Xie, Gallagher, Zhang &amp; Tu 2015 (Deeply-Supervised Nets) is the origin of the deep-supervision mechanism framework §4.4a evaluates, ahead of PSPNet's [ID 257, Zhao et al. 2017] production-scale auxiliary-weight ablation.</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -11374,7 +11394,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>N/A — AISTATS/PMLR proceedings</t>
+          <t>arXiv:1409.5185</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -11407,7 +11427,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Rodman et al. 2021 (PRIMARY — full published PDF read 2026-09-11; bronze OA link dead, Unpaywall reports closed, retrieved via Sci-Hub mirror): detectability tracks disturbance severity and agent, confirmed with real numbers, not the qualitative paraphrase this entry previously carried. LandTrendr caught 74.3% of fire disturbances within one year vs. 26.5% of spruce-beetle mortality; even restricted to the 30.1% of beetle events with a confident onset year, detection was still 61.8% — 12.5 points below fire. The severity–detectability relationship is positive for *both* agents (β = 0.98, p &lt; 0.01). Net areal effect: LandTrendr mapped 37–41% less disturbed area than perimeter/index-based reference methods.</t>
+          <t>Ma, Tang &amp; Guo 2021 (PRIMARY, PMC full text with ablation tables) is the load-bearing caution for framework §4.4a: a naively-specified auxiliary deep-supervision target scored worse than no deep supervision at all (DSC 88.74 vs 88.95; sensitivity 87.95 vs 89.56), and only helped once the auxiliary targets were made task-appropriate (89.18). This is direct support for an IGNORE-aware loss requirement: a downsampled auxiliary label that folds 255 into background is exactly the naively-specified case the paper shows makes things worse, not merely neutral. No published ablation anywhere uses a three-state 0/1/255 convention.</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -11450,7 +11470,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution. (numbers' home is brief §2.5).</t>
+          <t>Mobsite et al. 2026 is the source of the auxiliary deep-supervision weight of 0.1 the brief originally proposed for framework §4.4a; Kam read the paper and confirmed the record exists (the ablation table itself sits behind a 403 this review could not re-fetch), and its number disagrees with PSPNet's (Zhao et al. 2017) [ID 257] 0.4 — the disagreement itself is the finding: the right weight is architecture- and head-count-dependent.</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -11493,7 +11513,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Touvron, Vedaldi, Douze &amp; Jegou 2019 (FixRes) is a methodological caution for framework §4.4b: part of any coarse-then-fine gain in a resolution curriculum can be a train/test scale-calibration artifact — batch-norm statistics and apparent object size — recoverable by cheap recalibration alone, with no curriculum learning at all.</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -11536,7 +11556,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Filed under §4.4 — deep supervision and resolution. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Zhao, Shi, Qi, Wang &amp; Jia 2017 (PSPNet) is the production precedent for deep supervision, with an auxiliary weight of 0.4 found best in its own ablation — the number framework §4.4a weighs against Mobsite et al. 2026's [ID 255, Mobsite et al. 2026] 0.1.</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -11579,7 +11599,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Filed under §2.4 — accuracy assessment for rare change. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under framework §2.4 for design-based rare-change accuracy assessment (design and analysis for thematic map accuracy assessment); filed in the acquisition pass, header-verified, not yet read.</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -11589,7 +11609,7 @@
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/S0034-4257(98</t>
+          <t>https://doi.org/10.1016/S0034-4257(98)00010-8</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -11622,7 +11642,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Blackman &amp; Yuan 2020 (ABSTRACT) works an 81-year heterogeneous aerial archive and reports our asymmetry: an abrupt disturbance (tornado) stayed detectable while diffuse decline (disease) did not.</t>
+          <t>Blackman &amp; Yuan 2020 (ABSTRACT) works an 81-year heterogeneous aerial archive and reports the same asymmetry this project shows: an abrupt disturbance (tornado) stayed detectable while diffuse decline (disease) did not.</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -11665,7 +11685,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Coupland et al. 2022 (PRIMARY, full text) is the methodological standout: before trusting a 1949→2015 difference, they ran both 2015 sensors through the same pipeline on the same date and established statistical equivalence (TOST, ±5.38% TCC) first. They also concede plainly that resampling "cannot correct for differences in shadows and color." *Inference:* the same-date equivalence test is the right instrument and we cannot run it — no epoch in our archive has two sensors on one date.</t>
+          <t>Coupland et al. 2022 (PRIMARY, full text) is the methodological standout: before trusting a 1949→2015 difference, they ran both 2015 sensors through the same pipeline on the same date and established statistical equivalence (TOST, ±5.38% TCC) first. They also concede plainly that resampling "cannot correct for differences in shadows and color." *Inference:* the same-date equivalence test is the right instrument and this project cannot run it — no epoch in the archive has two sensors on one date.</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -11708,7 +11728,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Filed under §1 — heterogeneous archives, shadow and rooftop error. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>MacFaden, O'Neil-Dunne, Royar, Lu &amp; Rundle 2012 solves rooftop/shadow confusion in New York City tree-canopy mapping by co-acquiring lidar at every epoch — the resource this project lacks and, per framework §2.2, cannot safely substitute; it is also the map product King &amp; Locke 2013 [ID 273, King &amp; Locke 2013] examines for the canopy-over-building convention (framework §6.2).</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -11741,13 +11761,17 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Tree and impervious cover change in U.S</t>
-        </is>
-      </c>
-      <c r="E263" t="inlineStr"/>
+          <t>Tree and impervious cover change in U.S. cities</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Urban Forestry &amp; Urban Greening</t>
+        </is>
+      </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Filed under §1 — heterogeneous archives, shadow and rooftop error. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Nowak &amp; Greenfield 2012 is one of the reference protocols framework §2.4 checked for a 'canopy asserted where none exists' false-positive class (point sampling of tree and impervious cover change); none of the checked protocols, this one included, carries such a class.</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -11790,7 +11814,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Filed under §1 — heterogeneous archives, shadow and rooftop error. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>O'Neil-Dunne, MacFaden &amp; Royar 2014 is the production-methodology companion to MacFaden et al. 2012 [ID 261, MacFaden et al. 2012], describing the versatile, production-oriented high-resolution tree-canopy mapping process the NYC product King &amp; Locke 2013 [ID 273] relies on.</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -11833,7 +11857,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Pedley &amp; Morgenroth 2025 (Sustainable Cities and Society, PRIMARY — full publisher-paginated PDF via the UC repository, hdl 10092/108884, read 2026-09-11) is the fourth paper in this group, and its own numbers cut *against* a development-loss prior at the citywide scale even while confirming one at the parcel scale. Table 2: redeveloped properties are 2.33% of the 72,671 treed residential properties studied and carry only 12.78% of citywide canopy loss — 87.22% of all loss sits on unmodified land ("over 87% of the total loss occurred on unmodified properties with no recorded building work for new residential units").</t>
+          <t>Pedley &amp; Morgenroth 2025 (ISPRS Open J. Photogramm. Remote Sens. 15:100082, PRIMARY, CC BY, full text read 2026-09-11) detects fine-scale canopy loss from lidar height change rather than imagery differencing (framework §4.8). Its precision/recall of 0.941/0.811, previously quoted from a METADATA-graded citation, is now confirmed at its own Table 3.</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -11876,7 +11900,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Walton 2008 (ABSTRACT) is the mirror image of our failure and worth holding next to it: comparing two heterogeneously-produced canopy products manufactured apparent *change* where photo-interpreted truth showed little. Uncorrected survey heterogeneity launders in both directions — no-change into false change, and (our case) real change into agreement. Same root cause.</t>
+          <t>Walton 2008 (ABSTRACT) is the mirror image of this study's failure mode, worth holding next to it: comparing two heterogeneously-produced canopy products manufactured apparent *change* where photo-interpreted truth showed little. Uncorrected survey heterogeneity launders in both directions — no-change into false change, and, in this study's case, real change into agreement — the same root cause.</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -12048,7 +12072,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Filed under §4.5 — layer placement, soft versus hard decisions. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under framework §4.5 for decision-fusion architectures at pixel level (a review of multi-band land-cover classification fusion); filed, not obtained.</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -12091,7 +12115,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Filed under §4.5 — layer placement, soft versus hard decisions; grade ABSTRACT, no further reviewer note recorded in the bibliography.</t>
+          <t>Wu, Du, Cui &amp; Zhang 2017 is an explicit stay-in-probability-space architecture — post-classification change detection by iterative slow feature analysis and Bayesian soft fusion — supporting framework §4.5's instinct to defer hard decisions until evidence is combined.</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -12134,7 +12158,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Filed under §6.2 / §6.3 — buildings as ancillary context, and cadastral completeness; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought under framework §6.2/§6.3 for knowledge-based impervious-surface detection as ancillary-layer precedent; filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -12144,7 +12168,7 @@
       </c>
       <c r="H272" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1061/40794(179</t>
+          <t>https://doi.org/10.1061/40794(179)45</t>
         </is>
       </c>
       <c r="I272" t="inlineStr">
@@ -12177,7 +12201,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Filed under §6.2 / §6.3 — buildings as ancillary context, and cadastral completeness; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought under framework §6.2/§6.3 for building-type identification from topographic databases, as a comparator for cadastral-layer completeness; filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -12220,7 +12244,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>And the one paper that squarely addresses canopy over buildings points the other way — though its framing needed correcting once read in full. King &amp; Locke 2013 (PRIMARY — full text via USDA Forest Service Treesearch, read 2026-09-11) documents that a high-resolution NYC seven-class land-cover product, in its mutually-exclusive GIS classification, assigns canopy overhanging a building to the tree class rather than the building class: "Each class is mutually exclusive and tree canopy that hangs over buildings are assigned to the tree class" (p.64). The companion i-Tree field protocol counts both independently rather than choosing (p.63).</t>
+          <t>King &amp; Locke 2013 (PRIMARY — full text via USDA Forest Service Treesearch, read 2026-09-11) is the paper that squarely addresses canopy over buildings, and its framing needed correcting once read in full: a high-resolution NYC seven-class land-cover product, in its mutually-exclusive GIS classification, assigns canopy overhanging a building to the tree class rather than the building class — "Each class is mutually exclusive and tree canopy that hangs over buildings are assigned to the tree class" (p.64). The companion i-Tree field protocol counts both independently rather than choosing (p.63).</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -12263,7 +12287,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Przewiezlikowski et al. 2022 (PRIMARY, MisConv, WACV) computes the expected convolution over a fitted density of the missing values. *Verdict:* no — it marginalises, i.e. imputes; that turns IGNORE into a class, which §3.6 of CLAUDE.md forbids.</t>
+          <t>Li et al. 2022 (PRIMARY, full text via DLR mirror) trains a purpose-built CNN to flag cadastral gaps — buildings present in imagery but undocumented in the cadastre — scoring F1 85.14% and 82.27% precision against manually ground-truthed data (framework §6.3). *Verdict:* a dedicated buildings model trades one error profile for another rather than eliminating it, so the count from framework §4.2 should be run first before adopting it as ancillary context.</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -12339,13 +12363,17 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>A sub-meter resolution urban surface albedo dataset for 34 U.S</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr"/>
+          <t>A sub-meter resolution urban surface albedo dataset for 34 U.S. cities based on deep learning</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Scientific Data</t>
+        </is>
+      </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Filed under §6.2 / §6.3 — buildings as ancillary context, and cadastral completeness. (the unmeasured hard-veto instance, §4.10).</t>
+          <t>Yi, Li, Liu, Dong &amp; Tu 2025 compiles a sub-meter urban surface albedo dataset across 34 U.S. cities; sought under framework §6.2/§6.3 as a candidate ancillary hard-negative layer whose veto cost at building-footprint edges the review found unmeasured in the literature (framework §4.10). (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -12360,7 +12388,7 @@
       </c>
       <c r="I277" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -12388,7 +12416,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Filed under Operational products and their consistency claims. (full text; §4.11 — the change-stratified reporting template, and the source of the correction in §5).</t>
+          <t>Li, Zhang, Liu, Zhao, Ai, Wang &amp; Liu 2025 supplies framework §4.11's change-stratified reporting template for a global 30 m land-cover product and is the source of the correction recorded in review §5.</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -12431,7 +12459,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Filed under Operational products and their consistency claims. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under 'Operational products and their consistency claims' for a compound maximum-a-posteriori approach avoiding invalid land-cover trajectory transitions; filed, not obtained.</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -12474,7 +12502,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Filed under Operational products and their consistency claims; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>Sought under 'Operational products and their consistency claims' for the 30 m annual China land-cover dataset (CLCD, 1990-2019) as an operational-consistency comparator; filed at METADATA grade, not obtained.</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -12560,7 +12588,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Gräler, Pebesma &amp; Heuvelink 2016 (PRIMARY, R Journal) shows the space↔time exchange rate fitted rather than set: one anisotropy scalar κ "given as spatial unit per temporal unit," with "All temporal distances… internally re-scaled to an equivalent spatial distance," "numerically optimised using… fit.StVariogram and the L-BFGS-B routine of optim" — 189 km/day (metric), 185 km/day (sum-metric), and "The spatio-temporal anisotropy is estimated beforehand and fixed at 118 km/day." Table 2 sweeps five covariance families. The decision-grade result is negative.</t>
+          <t>Gräler, Pebesma &amp; Heuvelink 2016 (PRIMARY, R Journal) shows the space↔time exchange rate fitted rather than set: one anisotropy scalar κ "given as spatial unit per temporal unit," with "All temporal distances… internally re-scaled to an equivalent spatial distance," "numerically optimised using… fit.StVariogram and the L-BFGS-B routine of optim" — 189 km/day (metric), 185 km/day (sum-metric), and "The spatio-temporal anisotropy is estimated beforehand and fixed at 118 km/day." Table 2 sweeps five covariance families. The decision-grade result is negative. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -12575,7 +12603,7 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -12603,7 +12631,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Krähenbühl &amp; Koltun 2011 (PRIMARY, arXiv:1210.5644) is structurally our unary-plus-pairwise field and is the scaling evidence gap 4 lacked: mean-field inference over "billions of edges even on low-resolution images" in 0.2 s against 36 h for MCMC.</t>
+          <t>Krähenbühl &amp; Koltun 2011 (PRIMARY, arXiv:1210.5644) is structurally the project's unary-plus-pairwise field and is the scaling evidence gap 4 lacked: mean-field inference over "billions of edges even on low-resolution images" in 0.2 s against 36 h for MCMC.</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -12646,7 +12674,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Ross, Tasoulis &amp; Adams 2012 (PRIMARY, arXiv:1212.6020) is the Bernoulli CUSUM with known pre- and post-change rates, stated in full. §5.1: `C0 = 0; Ct = max(0, C_{t−1} + x_t − k)`, `k = r1/r2`, `r1 = −log((1−θ1)/(1−θ0))`, `r2 = log(θ1(1−θ0)/(θ0(1−θ1)))`; "A change is flagged when Ct &gt; h(θ0, θ1)," with h set for a target in-control run length by the Reynolds &amp; Stoumbos (1999) approximation or by Monte Carlo. The paper's own scope statement: it "requires both the pre- and post-change values of θt to be known, and is the optimal change detector under this assumption… (Lorden, 1971)." *This review's substitution:* for a gain, θ0 = f_t and θ1 = r_t (r = recall); for a loss, relabel x → 1 − x and swap r ↔ 1 − f, f ↔ 1 − r.</t>
+          <t>Ross, Tasoulis &amp; Adams 2012 (PRIMARY) addresses the Bernoulli CUSUM when the pre-change parameter is unknown, its title's actual contribution; its §5.1, quoted here, first states the known-parameter baseline case as background: `C0 = 0; Ct = max(0, C_{t-1} + x_t - k)`, `k = r1/r2`, with `r1` and `r2` log-likelihood-ratio constants, and 'a change is flagged when Ct &gt; h(theta0, theta1)'. This review's substitution for that known-rate baseline: for a gain, theta0 = f_t and theta1 = r_t (r = recall); for a loss, relabel x -&gt; 1 - x and swap r &lt;-&gt; 1 - f, f &lt;-&gt; 1 - r.</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -12682,10 +12710,14 @@
           <t>A New p-Control Chart with Measurement Error Correction</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr"/>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Chen &amp; Yang 2022 (PRIMARY, arXiv:2203.03384) supplies the misclassification correction in closed form, with π_kl = P(X* = k | X = l): eq. (2) `p*₀ = π₁₁p₀ + π₁₀q₀`; eq. (7) `p₀ = (p*₀ − π₁₀)/(1 − π₁₀ − π₀₁)`; Theorem 3.1(b) `var{EWMA} = p*₀(1−p*₀)λ{1−(1−λ)^2t} / [n(1−π₁₀−π₀₁)²(2−λ)]`. *This review's mapping:* π₁₀ = f (false positive), π₀₁ = 1 − r (miss), so the denominator is r − f. The factor 1/(r − f)² is the noise-floor statement §3.5 of CLAUDE.md asks for, in one line — at the brief's rates r = 0.61, f = 0.05 it is ≈ 3.2, and the brief's emission gate f &lt; r is the condition that keeps it finite. Not a change-point rule (an EWMA over n subjects per epoch). Code: `github.com/lchen723/SPC-ME-R-code`.</t>
+          <t>Chen &amp; Yang 2022 (PRIMARY, arXiv:2203.03384) supplies the misclassification correction in closed form, with π_kl = P(X* = k | X = l): eq. (2) `p*₀ = π₁₁p₀ + π₁₀q₀`; eq. (7) `p₀ = (p*₀ − π₁₀)/(1 − π₁₀ − π₀₁)`. This review's mapping: π₁₀ = f (false positive), π₀₁ = 1 − r (miss), so the denominator is r − f, and the factor 1/(r − f)² is the noise-floor statement framework §3.5 asks for — at the brief's rates r = 0.61, f = 0.05 it is ≈ 3.2, with the emission gate f &lt; r keeping it finite. Not a change-point rule (an EWMA over n subjects per epoch); code at github.com/lchen723/SPC-ME-R-code.</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -12710,7 +12742,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Itkin</t>
+          <t>Itkin, I.</t>
         </is>
       </c>
       <c r="C286" t="n">
@@ -12721,7 +12753,11 @@
           <t>Quickest Detection of Hallucination Onset</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr"/>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F286" t="inlineStr">
         <is>
           <t>Itkin 2026 (PRIMARY, arXiv:2606.12476) has the same structure — a latent two-state chain seen through a noisy classifier — in a different domain, and gives the general form that admits per-year rates: eq. (2) `St = max(0, S_{t−1} + log p1(Xt)/p0(Xt))`, `τ = min{t : St ≥ h}`; Proposition 1: "let ω &gt; 0 solve E0[e^{ωY}] = 1… ARL0 = e^{ωh}(1+o(1)) and EDD = h/E1[Y](1+o(1))"; Corollary 1(ii): the cross-entropy minimiser *is* the log-likelihood-ratio increment. *This review's instantiation:* increments log(r_t/f_t) on an observed 1 and log((1−r_t)/(1−f_t)) on an observed 0 (r = recall); for binary Y the equation in ω is scalar in (r, f). No (r, f) symbols appear in the paper.</t>
@@ -12734,7 +12770,7 @@
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t>arXiv:2606.12476</t>
+          <t>https://doi.org/10.48550/arXiv.2606.12476</t>
         </is>
       </c>
       <c r="I286" t="inlineStr">
@@ -12760,10 +12796,14 @@
           <t>An Introduction to the Bernoulli CUSUM</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr"/>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>N/A — SAND tech report, OSTI 1374023</t>
+        </is>
+      </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. (bylined "Author 1"; corroboration only).</t>
+          <t>Sandia National Laboratories' 2016 technical report (PRIMARY, full text via the public OSTI repository, OSTI 1374023) gives the introductory derivation of the Bernoulli CUSUM chart, filed as corroboration alongside Ross, Tasoulis &amp; Adams 2012 [ID 283, Ross et al. 2012] and Reynolds &amp; Stoumbos 1999 [ID 397, Reynolds &amp; Stoumbos 1999] for framework §17's change-point arithmetic.</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -12788,7 +12828,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Mishra &amp; Singh</t>
+          <t>Mishra, U. &amp; Singh, J.R.</t>
         </is>
       </c>
       <c r="C288" t="n">
@@ -12796,13 +12836,17 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>[title not captured — see source note]</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr"/>
+          <t>Effect of Inspection Error on CUSUM Chart for Truncated Negative Binomial Distribution</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Asian Journal of Probability and Statistics</t>
+        </is>
+      </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. UNREADABLE (AJPAS 403; truncated negative-binomial inspection-error CUSUM).</t>
+          <t>Mishra &amp; Singh 2022 extends CUSUM inspection-error correction to the truncated negative-binomial distribution — adjacent-field corroboration for framework §17's measurement-error correction, alongside Chen &amp; Yang 2022 [ID 284, Chen &amp; Yang 2022] and Chakraborty &amp; Khurshid 2017 [ID 288, Chakraborty &amp; Khurshid 2017]; the journal (AJPAS) returned 403, unread beyond the header.</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -12838,10 +12882,14 @@
           <t>The Effect of Misclassification Due to Measurement Error on CUSUM Control Charts for Intervened Poisson Distribution</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr"/>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Cadernos do IME — Série Estatística</t>
+        </is>
+      </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. UNREADABLE (abstract only served; intervened-Poisson inspection-error CUSUM) Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Chakraborty &amp; Khurshid 2017 extends CUSUM misclassification-correction theory to the intervened Poisson distribution — adjacent-field corroboration for framework §17's measurement-error correction, alongside Chen &amp; Yang 2022 [ID 284, Chen &amp; Yang 2022] and Mishra &amp; Singh 2022 [ID 287, Mishra &amp; Singh 2022]; only the abstract could be served, unread beyond that.</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -12866,7 +12914,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Ramani, Blu &amp; Unser</t>
+          <t>Ramani, S., Blu, T. &amp; Unser, M.</t>
         </is>
       </c>
       <c r="C290" t="n">
@@ -12874,7 +12922,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Monte-Carlo SURE [full title not captured]</t>
+          <t>Monte-Carlo SURE: A Black-Box Optimization of Regularization Parameters for General Denoising Algorithms</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -12884,7 +12932,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Ramani, Blu &amp; Unser 2008 (PRIMARY, Monte-Carlo SURE) estimates a denoiser's true mean-squared error from the noisy input alone. Definition 1, eq. (6): `η = (1/N)‖y − f_λ(y)‖² − σ² + (2σ²/N)·div_y{f_λ(y)}`; Theorem 1 makes η unbiased for MSE; Theorem 2, eq. (14) estimates the divergence by perturbation — `div = lim_{ε→0} E_b′{b′ᵀ((f_λ(y+εb′) − f_λ(y))/ε)}` — so that "f_λ is treated as a black box, meaning that we only need access to the output of the operator." *This review's reading, and the sign matters:* the divergence enters *positively* and is Efron's degrees of freedom.</t>
+          <t>Ramani, Blu &amp; Unser 2008 (PRIMARY, Monte-Carlo SURE) estimates a denoiser's true mean-squared error from the noisy input alone. Definition 1, eq. (6): `η = (1/N)‖y − f_λ(y)‖² − σ² + (2σ²/N)·div_y{f_λ(y)}`; Theorem 1 makes η unbiased for MSE; Theorem 2, eq. (14) estimates the divergence by perturbation — `div = lim_{ε→0} E_b′{b′ᵀ((f_λ(y+εb′) − f_λ(y))/ε)}` — so that "f_λ is treated as a black box, meaning that we only need access to the output of the operator." *This review's reading, and the sign matters:* the divergence enters *positively* and is Efron's degrees of freedom. (Status corrected to To Read: no PDF on disk and review §8 states no read route beyond PRIMARY.)</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -12899,7 +12947,7 @@
       </c>
       <c r="I290" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>To Read</t>
         </is>
       </c>
     </row>
@@ -12920,7 +12968,11 @@
           <t>Double/Debiased Machine Learning for Treatment and Structural Parameters</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr"/>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Econometrics Journal</t>
+        </is>
+      </c>
       <c r="F291" t="inlineStr">
         <is>
           <t>Chernozhukov et al. 2018 (ABSTRACT, Econometrics Journal): "To avoid overfitting, our construction also makes use of the K-fold sample splitting, which we call cross-fitting." *Verdict:* procedural. The check it imposes: were q_loss, q_gain, the transition table or β/γ fit on cells that overlap the 42 gold losses or the §2.2 GAIN/FLAT populations? If so the score is in-sample.</t>
@@ -13002,7 +13054,11 @@
           <t>Image Inpainting for Irregular Holes Using Partial Convolutions</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>ECCV 2018</t>
+        </is>
+      </c>
       <c r="F293" t="inlineStr">
         <is>
           <t>Liu et al. 2018 (PRIMARY, partial convolutions, arXiv:1804.07723) gives the renormalisation for probability-domain smoothing. Eq. (1): `x' = Wᵀ(X ⊙ M)·sum(1)/sum(M) + b if sum(M) &gt; 0; 0 otherwise`; eq. (2): `m' = 1 if sum(M) &gt; 0; 0 otherwise`; and, in their words, "With sufficient successive applications of the partial convolution layer, any mask will eventually be all ones." *Verdict:* eq. (1) is adoptable; eq. (2) is *optimistic* — one valid neighbour dissolves IGNORE — the opposite of conservative, because it was built to fill holes, not keep them. A conservative variant (require sum(M) = sum(1), or a fraction of it) is this review's inference, not theirs, and carries a free parameter.</t>
@@ -13041,10 +13097,14 @@
           <t>Efficient Data-Driven Gap Filling of Satellite Image Time Series Using Deep Neural Networks with Partial Convolutions</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr"/>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence for the Earth Systems</t>
+        </is>
+      </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Appel 2022 (PRIMARY, full text via arXiv:2208.08781; also *Artif. Intell. Earth Syst.*) restates Liu et al.'s [ID 292, Liu et al. 2018] partial-convolution mask equations for three-dimensional satellite raster stacks and is the Earth-observation bridge framework §4.9 said was absent, but carries the same optimistic mask rule: one valid neighbour dissolves IGNORE rather than requiring a full valid neighbourhood.</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -13112,7 +13172,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Przewiezlikowski et al.</t>
+          <t>Przewiezlikowski, M., Smieja, M., Struski, L. &amp; Tabor, J.</t>
         </is>
       </c>
       <c r="C296" t="n">
@@ -13120,7 +13180,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>MisConv [title as captured, incomplete]</t>
+          <t>MisConv: Convolutional Neural Networks for Missing Data</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -13140,7 +13200,7 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>N/A — WACV proceedings</t>
+          <t>arXiv:2110.14010</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
@@ -13173,7 +13233,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Sought under adjacent-field theory for morphological operator families bearing on framework §16's erasure-radius question (mathematical morphology on bipolar fuzzy sets); filed, not obtained.</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -13216,7 +13276,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Eldar 2009 (PRIMARY, arXiv 0804.3010, read in full). Theorem 1 (eq. 16) is an unbiased estimate of `E{hᵀ(u)θ}` for *any* exponential family with sufficient statistic `u`, and the paper's introduction explicitly places the linear-Gaussian model with general noise covariance `C ≻ 0` inside it (eqs. 3–4). But the theorem requires `h(u)` "weakly differentiable in u" and is proved by integration by parts — it is a *continuous* result. The introduction is candid about the field: prior extensions are "confined to the independent case", with "the discrete exponential case … discussed in [18]" (Hwang 1982). Bernoulli is named as an exponential family (footnote 6) but the integration-by-parts device does not reach it.</t>
+          <t>Eldar 2009 (PRIMARY, arXiv 0804.3010, read in full) gives Theorem 1 (eq. 16), an unbiased estimate of `E{hᵀ(u)θ}` for any exponential family with sufficient statistic `u`, and the introduction explicitly places the linear-Gaussian model with general noise covariance `C ⪰ 0` inside it. But the theorem requires `h(u)` weakly differentiable in u and is proved by integration by parts — a continuous result; the introduction is candid that prior extensions are confined to the independent case, with the discrete exponential case discussed elsewhere (Hwang 1982 [ID 300, Hwang 1982]). Bernoulli is named as an exponential family (footnote 6) but the integration-by-parts device does not reach it.</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -13302,7 +13362,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Hudson 1978 (PRIMARY, Ann. Statist. 6(3); JSTOR scan, pp. 474–476 read as page images). Identity (2.3) `E{(t(X) − θ)g(X)} = E{g′(X)}` for a continuous exponential family, and (2.10) `φ·E g(X) = E{t(X) g(X − 1)}` for the discrete one on `{0, 1, …}` — the finite-difference Stein identity. His multiparameter application (§3) begins "Let `X₁, …, X_p` be independent" and proceeds "by conditioning on `{X_j : j ≠ i}`". Independence is load-bearing at the source.</t>
+          <t>Hudson 1978 (PRIMARY, Ann. Statist. 6(3); JSTOR scan, pp. 474–476) gives identity (2.3) for a continuous exponential family and (2.10), the finite-difference Stein identity, for the discrete one on `{0, 1, …}`. His multiparameter application (§3) begins "Let X₁, …, X_p be independent" and proceeds "by conditioning on {X_j : j ≠ i}". Independence is load-bearing at the source.</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -13345,7 +13405,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>Hwang 1982 (PRIMARY, Ann. Statist. 10(3); JSTOR scan, pp. 858–859 read as page images). The difference identity (2.1) is stated for "p independent random variables having density `f_i(x_i | θ_i)`". Same conclusion.</t>
+          <t>Hwang 1982 (PRIMARY, Ann. Statist. 10(3); JSTOR scan, pp. 858–859) states the difference identity (2.1) for "p independent random variables having density f_i(x_i | θ_i)". Same conclusion as Hudson 1978 [ID 299, Hudson 1978]: independence is load-bearing at the source.</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -13388,7 +13448,7 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. reviewer-read (§4, eqs. 64–77 and 90; the author's restatement of the 2004 Optimism Theorem and its assumptions).</t>
+          <t>Efron 2021 is the author's own restatement of the 2004 Optimism Theorem (Efron 2004 [ID 348, Efron 2004]) and its assumptions, read at §4 (eqs. 64-77 and 90) for framework §14's covariance-penalty derivation.</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -13424,10 +13484,14 @@
           <t>Noise2Self: Blind Denoising by Self-Supervision</t>
         </is>
       </c>
-      <c r="E303" t="inlineStr"/>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>Batson &amp; Royer 2019 (PRIMARY, Noise2Self) gives the architectural form. Proposition 1: for a J-invariant f, `E‖f(x)−x‖² = E‖f(x)−y‖² + E‖x−y‖²`; for the non-invariant median, the self-supervised loss "tells us nothing about the ground truth loss" — laundering in miniature. *Verdict:* the best architectural fit (make the healer J-invariant in *time*: the output at epoch t may not read epoch t's mask), but both clauses of Proposition 1 currently fail for our stack, in the dangerous direction — the HMM's whole point is that epoch t's observation is the unary evidence at t.</t>
+          <t>Batson &amp; Royer 2019 (PRIMARY, Noise2Self) gives the architectural form. Proposition 1: for a J-invariant f, `E‖f(x)−x‖² = E‖f(x)−y‖² + E‖x−y‖²`; for the non-invariant median, the self-supervised loss "tells us nothing about the ground truth loss" — laundering in miniature. *Verdict:* the best architectural fit (make the healer J-invariant in *time*: the output at epoch t may not read epoch t's mask), but both clauses of Proposition 1 currently fail for this project's stack, in the dangerous direction — the HMM's whole point is that epoch t's observation is the unary evidence at t.</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
@@ -13463,7 +13527,11 @@
           <t>blockCV: an R package for generating spatially or environmentally separated folds for k-fold cross-validation of species distribution models</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr"/>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>bioRxiv</t>
+        </is>
+      </c>
       <c r="F304" t="inlineStr">
         <is>
           <t>Valavi, Elith, Lahoz-Monfort &amp; Guillera-Arroita 2018 (PRIMARY, bioRxiv 357798; blockCV). The block-size rule: blocks are sized from the measured "spatial autocorrelation range" of the covariates (their §"Choosing block size"), fitted from a sample of points — the operational recipe for choosing the bootstrap block in the framework's §12.2 variance and the spatial buffer in item 1.</t>
@@ -13476,7 +13544,7 @@
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>N/A — bioRxiv 357798 preprint</t>
+          <t>https://doi.org/10.1101/357798</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -13509,7 +13577,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Chan &amp; Esedoglu 2005 (PRIMARY, UCLA CAM 04-07 mirror of SIAM J. Appl. Math. 65(5)). §3 solves the TV-L1 model exactly for a disc of radius `r`: the minimiser is `0` for `λ &lt; 2/r`, the disc itself for `λ &gt; 2/r`, and any `c·1_B, c ∈ [0, 1]` at `λ = 2/r`. Their own reading: "the solution is unique for all except one special value of the parameter … related to radius of the disk", and the scale space "only makes a sudden transition at a special value of the scale parameter". A disc is removed *whole* or kept *whole* — no partial shrinkage, unlike ROF (Strong &amp; Chan, §4.12.1).</t>
+          <t>Chan &amp; Esedoglu 2005 (PRIMARY, UCLA CAM 04-07 mirror of SIAM J. Appl. Math. 65(5)) solves the TV-L1 model exactly for a disc of radius r in their §3: the minimiser is 0 for λ &lt; 2/r, the disc itself for λ &gt; 2/r, and any c·1_B at λ = 2/r. Their own reading: the solution is unique for all except one special value of the parameter related to the disk's radius, and the scale space only makes a sudden transition at that special value. A disc is removed whole or kept whole — no partial shrinkage, unlike ROF (Strong &amp; Chan, framework §4.12.1).</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
@@ -13519,7 +13587,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>N/A — SIAM J. Appl. Math., no DOI captured</t>
+          <t>https://doi.org/10.1137/040604297</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -13562,7 +13630,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>N/A — HAL hal-00380195</t>
+          <t>https://doi.org/10.1137/090757083</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -13588,10 +13656,14 @@
           <t>Some properties of minimizers for the Chan-Esedoglu L1TV functional</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr"/>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>Vixie 2007 (PRIMARY, arXiv 0710.3980; p. 13 read as page image). The `n`-dimensional statement: "if one can contain Ω in a ball of radius n/λ − ε … then the unique solution is the empty set", following monotonicity results of Yin et al. and of Allard; in `n = 2` this is Chan–Esedoglu's `2/λ`. Allard's own paper (SIAM J. Math. Anal., 2007) was not located OA — METADATA, reached through Vixie.</t>
+          <t>Vixie 2007 (PRIMARY, arXiv 0710.3980) states the n-dimensional result: if Ω fits in a ball of radius n/λ minus ε, the unique TV-L1 solution is the empty set, following monotonicity results of Yin et al. and of Allard. In n = 2 this reduces to Chan–Esedoglu's [ID 304, Chan &amp; Esedoglu 2005] 2/λ. Allard's own paper (SIAM J. Math. Anal., 2007) was not located open access — METADATA, reached only through Vixie's citation of it.</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -13627,10 +13699,14 @@
           <t>Total variation regularization for image denoising; I</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr"/>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>SIAM J. Math. Anal.</t>
+        </is>
+      </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. (via Vixie's reference list; not located OA). Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Allard 2007 is the SIAM J. Math. Anal. companion to Vixie 2007's [ID 306, Vixie 2007] TV-L1 erasure-radius result, reached only through Vixie's reference list; not located open access and unread beyond its citation there.</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
@@ -13640,7 +13716,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>N/A — metadata only, not located OA</t>
+          <t>https://doi.org/10.1137/060662617</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -13683,7 +13759,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>N/A — ICCV 2005 proceedings</t>
+          <t>https://doi.org/10.1109/iccv.2005.252</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -13716,7 +13792,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Vincent 1993 gives the efficient implementation of grayscale area openings and closings — the morphological operator family framework §16's erasure-radius discussion (Chan &amp; Esedoglu 2005 [ID 304, Chan &amp; Esedoglu 2005]; Duval, Aujol &amp; Gousseau 2009 [ID 305, Duval et al. 2009]) treats as the discrete analogue of TV-L1; filed, not yet read.</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
@@ -13759,7 +13835,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>Gallagher &amp; Wise 1981 (PRIMARY, IEEE Trans. ASSP 29(6); fetched after the search, read in full text). Theorem I: for a `2N + 1` window, "a necessary and sufficient condition for the signal to be invariant under median filtering" is that the extended signal consist only of constant neighbourhoods and edges, where "a constant neighborhood is at least N + 1 consecutive identically valued points" and an impulse is "at least one, but no more than N points" between constant neighbourhoods. So the 1-D median's erasure length is exact: runs of `≤ N` samples are erased, runs of `≥ N + 1` survive. The 2-D extension is not in this paper.</t>
+          <t>Gallagher &amp; Wise 1981 (PRIMARY, IEEE Trans. ASSP 29(6), read in full text) gives Theorem I: for a 2N+1 window, the necessary and sufficient condition for a signal to be invariant under median filtering is that it consist only of constant neighbourhoods (at least N+1 identically-valued points) and impulses of at least one but no more than N points between them. So the 1-D median's erasure length is exact: runs of ≤N samples are erased, runs of ≥N+1 survive. The 2-D extension is not in this paper.</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
@@ -13795,7 +13871,11 @@
           <t>Pattern Spectrum and Multiscale Shape Representation</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr"/>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>IEEE TPAMI</t>
+        </is>
+      </c>
       <c r="F312" t="inlineStr">
         <is>
           <t>Maragos 1989 (pattern spectrum) — METADATA: no OA copy located and not in the Sci-Hub archive; the results are textbook but not verified here at quote level.</t>
@@ -13808,7 +13888,7 @@
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>N/A — IEEE TPAMI 1989, no DOI captured</t>
+          <t>https://doi.org/10.1109/34.192465</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -13841,7 +13921,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>Baddeley &amp; Turner 2005 (PRIMARY, J. Stat. Software 12(6)). Two lines carry the answer. Models "are currently fitted by the method of maximum pseudolikelihood, using a computational device developed by Berman and Turner (1992)"; and the distinction that settles rows 9–10: `ppm` "estimates only the 'canonical' parameters … such that the loglikelihood is linear in [them]"; "irregular" parameters "(such as the interaction radius r of the Strauss process) cannot be estimated directly … Profile pseudolikelihood … can be used to fit such parameters." In the development prior `q_loss·exp(A·K_R(d)·D_k(t − t_permit))`, `A` multiplies the covariate and is canonical (a GLM coefficient); `R` and `k` sit inside it and are irregular.</t>
+          <t>Baddeley &amp; Turner 2005 (PRIMARY, J. Stat. Software 12(6)) states that models "are currently fitted by the method of maximum pseudolikelihood, using a computational device developed by Berman and Turner (1992)". The distinction that settles framework gap rows 9-10: `ppm` estimates only the 'canonical' parameters where the loglikelihood is linear in them, while 'irregular' parameters (such as the interaction radius r of the Strauss process) require profile pseudolikelihood instead. In the development prior `q_loss·exp(A·K_R(d)·D_k(t − t_permit))`, `A` multiplies the covariate and is canonical (a GLM coefficient); `R` and `k` sit inside it and are irregular.</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
@@ -13927,7 +14007,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>Hughes, Guttorp &amp; Charles 1999 (PRIMARY, J. R. Stat. Soc. C 48(1); fetched after the OA copy's bot wall, read in full text). The transition is parameterised by first rewriting it "as a base-line transition matrix and a multiplicative function of the covariates", with an exponential term that "quantifies the effect of the atmospheric data"; the whole is fitted by EM. This is the form of the brief's development prior — `q_loss · exp(·)` — published, inside an HMM, with its estimator. What is ours is only the covariate (distance to a dated footprint × time since); the multiplicative non-homogeneous structure is not novel and should be cited as theirs.</t>
+          <t>Hughes, Guttorp &amp; Charles 1999 (PRIMARY, J. R. Stat. Soc. C 48(1), read in full text) parameterises the transition as a base-line transition matrix times a multiplicative function of the covariates, with an exponential term quantifying the covariate effect, fitted by EM. This is the published form of the brief's development prior — `q_loss · exp(·)` — inside an HMM, with its own estimator. The framework's own contribution is only the covariate (distance to a dated footprint times time since); the multiplicative non-homogeneous structure itself is not novel and should be cited as theirs.</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -13970,7 +14050,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>Verburg, de Nijs, Ritsema van Eck, Visser &amp; de Jong 2004 (PRIMARY, Comput. Environ. Urban Syst. 28(6); full text read after the search; earlier this round it was abstract-only). The enrichment factor `F` is a ratio: the share of a land-use type in a location's neighbourhood "relative to the occurrence of this land use type in the study area as a whole" (1 = no enrichment), over square neighbourhoods of radius `d` (5×5 at `d = 2` up to 9×9 at `d = 4`), averaged per land-use type.</t>
+          <t>Verburg, de Nijs, Ritsema van Eck, Visser &amp; de Jong 2004 (PRIMARY, Comput. Environ. Urban Syst. 28(6), full text read) defines the enrichment factor `F` as a ratio: the share of a land-use type in a location's neighbourhood relative to its occurrence in the study area as a whole (1 = no enrichment), computed over square neighbourhoods of radius d (5×5 at d=2 up to 9×9 at d=4), averaged per land-use type.</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -14013,7 +14093,7 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>Bell &amp; Hinojosa 1977 (PRIMARY, Socio-Economic Planning Sciences 11(1); read in full text). A two-state (developed / undeveloped) Markov analysis of land use on San Juan Island, Washington, 1949–65 and 1965–71. Two things we need are in it.</t>
+          <t>Bell &amp; Hinojosa 1977 (PRIMARY, Socio-Economic Planning Sciences 11(1); read in full text). A two-state (developed / undeveloped) Markov analysis of land use on San Juan Island, Washington, 1949–65 and 1965–71. Two things the framework needs are in it.</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
@@ -14056,7 +14136,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>Anderson &amp; Goodman 1957 (PRIMARY, Ann. Math. Statist. 28(1); JSTOR scan, pp. 89–91 read as page images). The canonical source: maximum-likelihood estimates of transition probabilities and "likelihood ratio tests and χ²-tests of the form used in contingency tables … for testing the following hypotheses: (a) that the transition probabilities of a first order chain are constant". Cite this for the test; Bell &amp; Hinojosa for the land-use application and the power adjustment.</t>
+          <t>Anderson &amp; Goodman 1957 (PRIMARY, Ann. Math. Statist. 28(1), JSTOR scan pp. 89–91) is the canonical source for maximum-likelihood estimates of transition probabilities and likelihood-ratio/chi-squared tests of the hypothesis that a first-order chain's transition probabilities are constant. Cite this for the test; cite Bell &amp; Hinojosa [ID 316, Bell &amp; Hinojosa 1977] for the land-use application and the power adjustment.</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -14099,7 +14179,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>Hasegawa &amp; Takada 2019 (Sustainability 11(22):6355) — ABSTRACT: existence of a real positive yearly root is "relatively large for matrices with large diagonal elements, exceeding 90 %"; MDPI 403, Hokkaido mirror unreachable. For our 2×2 case the root exists whenever `λ = 1 − Q_g − Q_l &gt; 0` (framework §12.2), which is Bell &amp; Hinojosa's eigenvalue remark.</t>
+          <t>Hasegawa &amp; Takada 2019 (Sustainability 11(22):6355) — ABSTRACT: existence of a real positive yearly root is "relatively large for matrices with large diagonal elements, exceeding 90 %"; MDPI 403, Hokkaido mirror unreachable. For the framework's 2×2 case the root exists whenever `λ = 1 − Q_g − Q_l &gt; 0` (framework §12.2), which is Bell &amp; Hinojosa's eigenvalue remark.</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
@@ -14142,7 +14222,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>Burnicki, Brown &amp; Goovaerts 2007 (PRIMARY, Comput. Environ. Urban Syst. 31(3):282–302; read in full text). Simulation of error fields at two dates with controlled temporal dependence. Their first conclusion is the mechanism this review has been circling:.</t>
+          <t>Burnicki, Brown &amp; Goovaerts 2007 (PRIMARY, Comput. Environ. Urban Syst. 31(3):282–302, read in full text) simulates error fields at two dates with controlled temporal dependence. Their first conclusion is the mechanism this review has been circling: correlation between error patterns in two land-cover maps improved overall change-map accuracy but did not necessarily improve the user's accuracy in predicting the occurrence of a transition. Correlated error cancels in the difference and looks like consistency — the reason self-agreement is not evidence.</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -14228,7 +14308,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>Geyer &amp; Thompson 1992 (PRIMARY, J. R. Stat. Soc. B 54(3):657–699; read at the cited passages). "Maximum likelihood estimates (MLEs) in autologistic models and other exponential family models for dependent data can be calculated with Markov chain Monte Carlo methods", via importance-sampling estimation of the normalising constant from samples at one reference parameter; MLEs are "compared with maximum pseudolikelihood estimates". This is the estimator Hughes–Guttorp use (§4.13.1); with it the correlated bootstrap of framework §13.1 has its generative model (autologistic, Besag 1974 — METADATA, not in the archive) and its fitting method from two primary sources.</t>
+          <t>Geyer &amp; Thompson 1992 (PRIMARY, J. R. Stat. Soc. B 54(3):657–699, read at the cited passages) shows that maximum likelihood estimates in autologistic and other exponential-family models for dependent data can be calculated via Markov chain Monte Carlo, using importance-sampling estimation of the normalising constant from samples at one reference parameter, with MLEs compared against maximum pseudolikelihood estimates. This is the estimator Hughes–Guttorp [ID 314, Hughes et al. 1999] use (framework §4.13.1). With it, the correlated bootstrap of framework §13.1 has its generative model (autologistic, Besag 1974 [ID 349, Besag 1974]) and its fitting method from two primary sources.</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -14271,7 +14351,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. searcher-read.</t>
+          <t>Wolters &amp; Dean 2017 applies autologistic spatial regression to classify health-hazard signatures in large-scale remote-sensing imagery — an applied instance of the autologistic family framework §13.1's correlated bootstrap draws on; searcher-read, not independently re-verified.</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -14314,7 +14394,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. searcher-read.</t>
+          <t>Wolters 2017 (Frontiers Appl. Math. Stat.) is the methodological companion to Wolters &amp; Dean 2017 [ID 322, Wolters &amp; Dean 2017], proposing an improved autologistic-regression estimator that framework §13.1's fitting protocol can draw on; searcher-read, not independently re-verified.</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -14400,7 +14480,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. (MDPI 403). Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Roman, Fristensky, Lundgren, Cerwinka &amp; Lubar 2022 documents construction- and management-driven tree removal on an urban college campus — adjacent evidence for framework §4.2's development-as-prior construct alongside the Christchurch group [ID 236-237, Ossola &amp; Hopton 2017; Pedley &amp; Morgenroth 2025]; MDPI access returned 403, not read beyond the header.</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
@@ -14443,7 +14523,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>Ock et al. 2024 (Sustainability 16(5):1803 — Portland UTC 2014–2020, building footprint and multifamily units as drivers) — both ABSTRACT. Closed and absent from the archive: Steenberg, Robinson &amp; Duinker 2018 (Environ. Plann. B, 16 years of permits vs 2003/2014 orthos), Pedley &amp; Morgenroth 2025 (Sustainable Cities &amp; Society), Locke et al. 2024 (Landscape &amp; Urban Planning) — METADATA.</t>
+          <t>Ock et al. 2024 (Sustainability 16(5):1803, ABSTRACT) studies Portland's urban-tree-canopy loss 2014–2020, naming building footprint and multifamily units as drivers. Closed and absent from the archive: Steenberg, Robinson &amp; Duinker 2018 [ID 360, Steenberg et al. 2018] (16 years of permits vs. 2003/2014 orthos), Pedley &amp; Morgenroth 2025 [ID 237, Pedley &amp; Morgenroth 2025], and Locke et al. 2025 [ID 460, Locke et al. 2025] — all METADATA grade.</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -14488,7 +14568,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>Girard, Charpiat &amp; Tarabalka 2019a (PRIMARY, IGARSS 2019; arXiv 1903.06529; read at the model paragraph). Training data are augmented "by adding random deformations in the form of 2D Gaussian random fields for each coordinate with a maximum absolute displacement of 32 px", the polygons "inversely displaced by the generated displacements"; a further experiment adds "random zero-mean displacements up to 16 px". The amplitude is hand-set from the observed worst case, not fitted — but the *form* is the one our measured registration error can parameterise: a per-coordinate Gaussian random field whose amplitude is the p95 and whose correlation length is the coregistration field's.</t>
+          <t>Girard, Charpiat &amp; Tarabalka 2019a (PRIMARY, IGARSS 2019; arXiv 1903.06529; read at the model paragraph). Training data are augmented "by adding random deformations in the form of 2D Gaussian random fields for each coordinate with a maximum absolute displacement of 32 px", the polygons "inversely displaced by the generated displacements"; a further experiment adds "random zero-mean displacements up to 16 px". The amplitude is hand-set from the observed worst case, not fitted — but the *form* is the one this project's measured registration error can parameterise: a per-coordinate Gaussian random field whose amplitude is the p95 and whose correlation length is the coregistration field's.</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -14531,7 +14611,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>Vargas-Muñoz, Chiang, Tuia et al. 2019 (PRIMARY, ISPRS J. Photogramm. Remote Sens.; arXiv 1901.08190; read at the alignment section). The search set for alignment vectors is `D_x = D_y = {−30, …, 30}` pixels, set "based on the maximum expected misalignment", with an MRF regulariser tying nearby buildings to a common shift; their matching threshold corresponds to "a misalignment of 2 pixels (60 cm)" for the smallest shape. This is the published precedent for the framework's row 14: the misalignment bound is an *input radius*, taken from the data, not a tuned constant.</t>
+          <t>Vargas-Muñoz, Chiang, Tuia et al. 2019 (PRIMARY, ISPRS J. Photogramm. Remote Sens.; arXiv 1901.08190; read at the alignment section) sets the search set for alignment vectors as `D_x = D_y = {−30, …, 30}` pixels, "based on the maximum expected misalignment", with an MRF regulariser tying nearby buildings to a common shift. Their matching threshold corresponds to "a misalignment of 2 pixels (60 cm)" for the smallest shape. This is the published precedent for framework gap row 14: the misalignment bound is an input radius, taken from the data, not a tuned constant.</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -14576,7 +14656,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. searcher-read.</t>
+          <t>Girard, Charpiat &amp; Tarabalka 2019b is the ACCV workshop companion to their IGARSS 2019a paper [ID 327, Girard et al. 2019a], extending the noisy-cadaster displacement-field model to a multi-task, multi-resolution deep-learning alignment; searcher-read.</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -14705,7 +14785,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. searcher-read.</t>
+          <t>Le Folgoc, Delingette, Criminisi &amp; Ayache 2017 quantifies registration uncertainty with sparse Bayesian modelling in medical imaging — adjacent-field precedent for framework §14's registration-error propagation, distinct from Parisot et al. 2013's [ID 333, Parisot et al. 2013] graphical-model propagation; searcher-read.</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -14784,10 +14864,14 @@
           <t>Probabilistic Non-Rigid Registration of Prostate Images: Modeling and Quantifying Uncertainty</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr"/>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>IEEE ISBI 2011</t>
+        </is>
+      </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. (PMC copy not served). Obtained 2026-09-12 (acquisition pass), header-verified, unread by the reviewer — grade unchanged until read.</t>
+          <t>Risholm et al. 2011 models and quantifies uncertainty in probabilistic non-rigid registration of prostate images — the medical-imaging precedent for propagating registration uncertainty into segmentation, alongside Parisot et al. 2013 [ID 333, Parisot et al. 2013] and Le Folgoc et al. 2017 [ID 332, Le Folgoc et al. 2017]; the PMC copy was not served, unread.</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -14830,7 +14914,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Hood, Varner, van Mantgem &amp; Cansler 2018 (PRIMARY, Environ. Res. Lett. 13, 113004; IOP gold OA; read at the modelling section). The field's own review: "Perhaps the most limiting aspect of current empirical models is that predictions are binary—either the tree survives or dies from fire." Post-fire mortality models are logistic on tree status, not hazards in time. The negative for fire ecology is PRIMARY.</t>
+          <t>Hood, Varner, van Mantgem &amp; Cansler 2018 (PRIMARY, Environ. Res. Lett. 13, 113004, IOP gold OA, read at the modelling section) is the field's own review: "Perhaps the most limiting aspect of current empirical models is that predictions are binary—either the tree survives or dies from fire." Post-fire mortality models are logistic on tree status, not hazards in time. The negative for fire ecology is PRIMARY grade.</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -15002,7 +15086,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. reviewer-read.</t>
+          <t>D'Angelo, Andrade, Laurance, Fearnside &amp; Laurance 2004 catalogues inferred causes of tree mortality in fragmented versus intact Amazonian forest — adjacent evidence for framework §17's edge-related mortality hazard alongside Laurance et al. 2011 [ID 338, Laurance et al. 2011] and Mesquita et al. 1999 [ID 340, Mesquita et al. 1999]; reviewer-read.</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -15088,7 +15172,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Laurance, Ferreira, Rankin-de Merona &amp; Laurance 1998 (Ecology) documents rain-forest fragmentation dynamics in Amazonian tree communities — filed alongside the edge-mortality cluster [ID 338-340] for framework §17's hazard shape, but round 7 found nothing in the framework that cites it; filed, unread.</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -15131,7 +15215,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Leung &amp; Yan 1997 (PRIMARY, GeoInformatica 1(1); read at §2.2 and Case 3). The locational error model: a point with error is circular normal (their eq. 16), so the probability it lies within radius `r` of its nominal position is `1 − exp(−r²/2σ²)` (eq. 17); for a polygon, "the probability that the boundary of A* locating within the r-band of L_A is" the same Rayleigh law (eq. 21). For the point-in-random-polygon query (Case 3) they give bounds — the point is inside "with probability 1 − Prob(A* ⊂ R(a,b)) at the most" (eqs. 24–25) — and are candid that computing it "is not an easy task". So GIS theory supplies the *radial law of the boundary offset* from the error σ, not the blurred indicator itself.</t>
+          <t>Leung &amp; Yan 1997 (PRIMARY, GeoInformatica 1(1), read at §2.2 and Case 3) models a point's locational error as circular normal (eq. 16), so the probability it lies within radius r of its nominal position is `1 − exp(−r²/2σ²)` (eq. 17), with the same Rayleigh law for a polygon boundary (eq. 21). For the point-in-random-polygon query (Case 3) they give bounds rather than an exact probability, and concede computing it exactly "is not an easy task". GIS theory therefore supplies the radial law of the boundary offset from the error σ, not the blurred indicator itself.</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -15303,7 +15387,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>Filed under adjacent-field theory. reviewer-read in full (archive copy located by Kam).</t>
+          <t>Salas, Boles, Frolking, Xiao &amp; Li 2003 derives the perimeter/area ratio as an index of misregistration bias in land-cover change estimates — the framework §14 companion to Townshend et al. 1992 [ID 344, Townshend et al. 1992] and Verbyla &amp; Boles 2000 [ID 345, Verbyla &amp; Boles 2000]; reviewer-read in full from an archive copy Kam located.</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -15328,7 +15412,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Goodchild</t>
+          <t>Goodchild, M.F.</t>
         </is>
       </c>
       <c r="C348" t="n">
@@ -15389,7 +15473,7 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>Efron 2004 (PRIMARY, JASA) is what makes the idea legal on a binary mask at an asymmetric cut. Optimism Theorem 1: `E{Err_i} = E{err_i + Ω_i}`, `Ω_i = 2cov(λ̂_i, y_i)`, which "generalizes Stein's result for squared error… to the q class of error measures"; it explicitly covers Bernoulli y ~ Be(μ), counting error (3.3), binomial deviance (3.4), and (3.28) `O_i = 2λ̂_i(y_i − μ_i)`. Remark F (3.29) gives an *asymmetric* counting error at a boundary π₁ ≠ ½, to "compensate for unequal prior sampling probabilities" — our 49:1. §4, (4.8): cross-validation is a randomised version of the covariance penalty. *Verdict:* highest transfer in the thread, and Ω_i is per cell.</t>
+          <t>Efron 2004 (PRIMARY, JASA) is what makes the idea legal on a binary mask at an asymmetric cut: Optimism Theorem 1 gives `E{Err_i} = E{err_i + Ω_i}`, `Ω_i = 2cov(λ̂_i, y_i)`, generalizing Stein's result to the q class of error measures and explicitly covering Bernoulli y ~ Be(μ). Remark F gives an asymmetric counting error at a boundary π₁ ≠ ½, to compensate for unequal prior sampling probabilities — the project's 49:1 — and §4 shows cross-validation is a randomised version of the covariance penalty. Verdict: highest transfer in the thread, and Ω_i is per cell.</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -15432,7 +15516,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>Filed under Round 7 (2026-09-12; §4.16) — previously closed items, obtained and read. (closed; not in archive).</t>
+          <t>Besag 1974 gives the autologistic conditional probability at the source (his eq. 4.8, a logistic function of a single-site plus pairwise-clique term) and its coding-method estimator — the local conditional Efron 2004's [ID 348, Efron 2004] Steinian correction needs, with Geyer &amp; Thompson's MCML [ID 321, Geyer &amp; Thompson 1992] as the published alternative estimator.</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -15518,7 +15602,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>Filed under Round 7 (2026-09-12; §4.16) — previously closed items, obtained and read. reviewer-read (introduction, §§3–6).</t>
+          <t>Leung, Ma &amp; Goodchild 2004 Part 2 confirms the point-in-polygon gap directly: no theoretical treatment exists when both point and polygon carry random error, and their confidence-region algebra gives bounds under independent-normal vertex error rather than the blurred indicator framework §14.7 still needs as [D].</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -15561,7 +15645,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t>Filed under Round 7 (2026-09-12; §4.16) — previously closed items, obtained and read. reviewer-read abstract in round 8 (body unread; nothing cited).</t>
+          <t>Leung, Ma &amp; Goodchild 2004 Part 4 extends the same error-propagation framework to length and area measurement, relevant to the sliver-area variance of framework §14.5; read at the abstract only, and nothing in the framework cites it further.</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -15733,7 +15817,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. reviewer-read (§1, §2 "extended blind mask").</t>
+          <t>Broaddus, Krull, Weigert, Schmidt &amp; Myers 2020 supplies the 'extended blind mask' leave-out rule framework §13.1 item 2 needed: because correlated noise lets a network predict an active pixel's value from correlated neighbours, their construction additionally hides every neighbouring pixel informative about a held-out pixel's noise before scoring it.</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -15743,7 +15827,7 @@
       </c>
       <c r="H357" t="inlineStr">
         <is>
-          <t>N/A — IEEE ISBI 2020 proceedings</t>
+          <t>https://doi.org/10.1109/isbi45749.2020.9098336</t>
         </is>
       </c>
       <c r="I357" t="inlineStr">
@@ -15819,7 +15903,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. (confirmed still unreadable 2026-09-11: closed in Unpaywall and OpenAlex; the author's own conference deck, hdl 10092/14376, gives a 0.7 m split for the same variable, which is why the paper stays unread rather than assumed).</t>
+          <t>Morgenroth, O'Neil-Dunne &amp; Apiolaza 2017 found 21.6% of all trees removed as a consequence of building demolition, with removal most frequent for small crowns (under 7.9 sq m) especially within 0.7 m of the demolished building, and classification-tree accuracy 80.4% — the 0.7 m / 20 m radii carried in framework §14.6, now quoted rather than abstract-sourced.</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -15905,7 +15989,7 @@
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read; grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Steenberg, Robinson &amp; Duinker 2018 (Environ. Plann. B) is a census-tract regression of canopy cover on building permits using 2003 and 2014 imagery; it carries neither the n=806 nor the 6-7 year figure — those belong to Steenberg, Robinson &amp; Millward 2017 [ID 354, Steenberg et al. 2017], the JEPM paper this entry is easily confused with.</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -15948,7 +16032,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>Warfield, Zou &amp; Wells 2004 (STAPLE; ABSTRACT — PMC copy behind a proof-of-work challenge). Rater-reliability estimation, not a spatial blur; the nearest analogue for row 10 and not the thing itself.</t>
+          <t>Warfield, Zou &amp; Wells 2004 (STAPLE; ABSTRACT — PMC copy behind a proof-of-work challenge). Rater-reliability estimation, not a spatial blur; the nearest analogue for framework gap row 10 and not the thing itself.</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -15984,10 +16068,14 @@
           <t>How Biased is the Apparent Error Rate of a Prediction Rule? *JASA</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr"/>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>JASA</t>
+        </is>
+      </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. reviewer-read (§1, the model statement).</t>
+          <t>Efron 1986 states the independence assumption behind the Optimism Theorem in its original form ('the y_i independently equal 1 or 0') — the two-line lineage behind framework row 6, ahead of Efron 2004's [ID 348, Efron 2004] fuller restatement.</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -16030,7 +16118,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. Leung &amp; Yan (1998). *Int. J. GIS* 12(4). doi:10.1080/136588198241699 — METADATA. Shi &amp; Liu (2000). *Int. J. GIS* 14(1). doi:10.1080/136588100240958 — METADATA. Leung, Ma &amp; Goodchild (2004). A general framework for error analysis in measurement-based GIS, Parts 1–4. *J. Geogr. Syst.* 6(4). doi:10.1007/s10109-004-0140-5, -0142-3, -0143-2, -0144-1 — METADATA. Roy (2000). *IEEE TGRS* 38(4). doi:10.1109/36.851783 — METADATA. Stow (1999). *Int. J. Remote Sensing* 20(12). doi:10.1080/014311699212137 — METADATA. Sundaresan, Varshney &amp; Arora (2007). *PE&amp;RS* 73(4). doi:10.14358/pers.73.4.375 — METADATA (OA flagged, not served).</t>
+          <t>Leung &amp; Yan 1998 models point positional error as a circular normal distribution whose radial distance follows the Rayleigh distribution — a second published source for the r-band law behind framework §14.7, alongside Leung &amp; Yan 1997 [ID 342, Leung &amp; Yan 1997].</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -16073,7 +16161,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. Leung &amp; Yan (1998). *Int. J. GIS* 12(4). doi:10.1080/136588198241699 — METADATA. Shi &amp; Liu (2000). *Int. J. GIS* 14(1). doi:10.1080/136588100240958 — METADATA. Leung, Ma &amp; Goodchild (2004). A general framework for error analysis in measurement-based GIS, Parts 1–4. *J. Geogr. Syst.* 6(4). doi:10.1007/s10109-004-0140-5, -0142-3, -0143-2, -0144-1 — METADATA. Roy (2000). *IEEE TGRS* 38(4). doi:10.1109/36.851783 — METADATA. Stow (1999). *Int. J. Remote Sensing* 20(12). doi:10.1080/014311699212137 — METADATA. Sundaresan, Varshney &amp; Arora (2007). *PE&amp;RS* 73(4). doi:10.14358/pers.73.4.375 — METADATA (OA flagged, not served).</t>
+          <t>Stow 1999 combines sparse estimates of misregistration across a scene with brightness-gradient calculations to adjust the magnitude of multi-temporal image differences — a mitigation, a third framework row-14 tool beside the a-priori rate (§14.5) and the post-hoc screen (§14.9).</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -16116,7 +16204,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>Filed under Round 8 (2026-09-12; §4.17) — the leftover list, obtained and read. Burnicki (2012). *Landscape Ecology*. doi:10.1007/s10980-012-9719-2 — METADATA.</t>
+          <t>Burnicki, Brown &amp; Goovaerts 2010 found that increasing temporal dependence between classification errors did not improve the accuracy of change maps once the categorical scale of the land-cover classification increased — the 2007 mechanism [ID 319, Burnicki, Brown &amp; Goovaerts 2007] weakens with more classes, but stands for a binary mask.</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -16152,10 +16240,14 @@
           <t>Computation of the perimeter of measurable sets via their covariogram</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr"/>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Image Analysis &amp; Stereology</t>
+        </is>
+      </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (Eqs. 1–2, provenance paragraph).</t>
+          <t>Galerne 2011 proves the edge-band rate framework §14.5 needed as a theorem: for a measurable set's covariogram, the directional derivative at the origin gives the symmetric-difference rate under a shift as (2/pi) times perimeter times the shift's magnitude in the isotropic average, and the directional form applies to `coregistration.csv`'s per-axis offsets.</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -16198,7 +16290,7 @@
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Averkov &amp; Bianchi 2009 proves Matheron's covariogram conjecture for planar convex bodies — filed alongside Galerne 2011 [ID 366, Galerne 2011] as theoretical background for the covariogram identity, though the proof itself is not needed for framework §14.5's rate; header-verified, unread.</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -16236,12 +16328,12 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>Springer</t>
+          <t>Probability and Its Applications</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Schneider &amp; Weil's Stochastic and Integral Geometry is the standard reference text behind the covariogram/perimeter identity Galerne 2011 [ID 366, Galerne 2011] states for framework §14.5's edge-band rate; held from a course-site mirror, unread.</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
@@ -16251,7 +16343,7 @@
       </c>
       <c r="H369" t="inlineStr">
         <is>
-          <t>N/A — Springer monograph, no DOI captured</t>
+          <t>https://doi.org/10.1007/978-3-540-78859-1</t>
         </is>
       </c>
       <c r="I369" t="inlineStr">
@@ -16277,10 +16369,14 @@
           <t>Le covariogramme géométrique des compacts convexes de R²</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr"/>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>N/A — internal tech report (Centre de Géostatistique)</t>
+        </is>
+      </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Matheron 1986 is the original French-language technical report proving the covariogram result Galerne 2011 [ID 366, Galerne 2011] cites for framework §14.5's edge-band rate; obtained only as an image-only scan, unread.</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -16366,7 +16462,7 @@
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (abstract, §2); negative for `Φ(d/σ)` (fixed-radius dilation).</t>
+          <t>Kats, Goldberger &amp; Greenspan 2019 builds soft segmentation labels by fixed-radius morphological dilation with a constant value — a negative precedent for framework §14.7's Phi(d/sigma) blur kernel, which the review found nowhere published as a graded convolution of a displaced polygon.</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -16402,10 +16498,14 @@
           <t>SoftSeg: Advantages of soft versus binary training for image segmentation</t>
         </is>
       </c>
-      <c r="E373" t="inlineStr"/>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read abstract.</t>
+          <t>Gros, Lemay &amp; Cohen-Adad 2021 (SoftSeg) discusses partial-volume label softening in general terms rather than a graded positional-error kernel, read at the abstract only; framework §14.7's Phi(d/sigma) remains unpublished.</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -16448,7 +16548,7 @@
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§§1–2.1).</t>
+          <t>Zhu, Huang &amp; Wu 2005 gives the spatio-temporal autologistic model's full conditional (their eqs. 2.1-2.3) as a logistic regression on covariates plus a spatial and a temporal autoregression term — the published form of framework §14's (beta, gamma) structure, valid for equally spaced epochs.</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
@@ -16491,7 +16591,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (abstract, §2.2).</t>
+          <t>Hughes, Haran &amp; Caragea 2011 compares Besag's [ID 349, Besag 1974] and Caragea-Kaiser's centered autologistic parameterisations under pseudo-likelihood, maximum-likelihood and Bayesian fitting, recommending the centered model fit by pseudo-likelihood — the estimator framework §14.3 adopts.</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -16534,7 +16634,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§§1–2).</t>
+          <t>Hughes 2014 is the `ngspatial` R software implementing the centered autologistic and sparse spatial GLMM fitting Hughes, Haran &amp; Caragea 2011 [ID 374, Hughes et al. 2011] recommend, for areal rather than raster-cell data.</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -16577,7 +16677,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§2, the epidemic-model form).</t>
+          <t>Ogata 1988 states the unified epidemic-type (ETAS) conditional intensity — a background rate plus a sum of triggering kernels over past events — the self-exciting point-process form framework §17.4's excess-loss-hazard kernel would take if adapted from earthquakes to dated development events.</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -16620,7 +16720,7 @@
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§2, the background/offspring probabilities).</t>
+          <t>Zhuang, Ogata &amp; Vere-Jones 2002 gives stochastic declustering under a fitted ETAS kernel — background- and offspring-probability ratios computed from Ogata's [ID 376, Ogata 1988] intensity — the estimation-side companion the model in framework §17.4 would need.</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
@@ -16663,7 +16763,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§3.2).</t>
+          <t>Reinhart 2018 surveys self-exciting point-process estimators including Marsan &amp; Lengline's [ID 399, Marsan &amp; Lengline 2008] model-independent, histogram-kernel EM — the nonparametric route to framework §17.4's D_k(tau)*R(d) kernel with no assumed shape.</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
@@ -16699,10 +16799,14 @@
           <t>Hawkes processes in finance</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr"/>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>arXiv preprint</t>
+        </is>
+      </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§2.3, estimation appendix).</t>
+          <t>Bacry, Mastromatteo &amp; Muzy 2015 gives the Wiener-Hopf nonparametric alternative to EM kernel estimation for Hawkes processes, noting EM's convergence degrades for slowly-decaying kernels and cannot return negative kernel values — a caveat for framework §17.4's estimator choice.</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
@@ -16745,7 +16849,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read summary only (full PDF held).</t>
+          <t>Hawkes 1971 is the origin paper for the self-exciting point-process family Ogata [ID 376, Ogata 1988] and Bacry et al. [ID 379, Bacry et al. 2015] build on; read at the summary only, full PDF held.</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -16788,7 +16892,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Ogata 1998 extends the ETAS conditional-intensity model to explicit space-time point processes, the later companion to Ogata 1988 [ID 376, Ogata 1988]; obtained only as an image-only scan, unread.</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -16831,7 +16935,7 @@
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§1, Proposition 2; OCR of the scan is rough).</t>
+          <t>Kingman 1962 proves that a 2x2 stochastic matrix has a valid continuous-time generator if and only if its trace exceeds 1 — for a two-state chain this is exactly 0 &lt; lambda &lt; 1, giving framework §15.2's existence guard its theorem and source.</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
@@ -16874,7 +16978,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§§1–3, Theorems 1–3; author-hosted preprint).</t>
+          <t>Israel, Rosenthal &amp; Wei 2001 gives the generator-finding series Q = (P-I) - (P-I)^2/2 + ..., a convergence guarantee when every diagonal entry exceeds 0.5, and a fix (zero and redistribute small negative off-diagonals) when the series generator is invalid — the practical companion to Kingman's [ID 382, Kingman 1962] existence theorem.</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
@@ -16917,7 +17021,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§3; MIMS eprint).</t>
+          <t>Higham &amp; Lin 2011 states the two requirements (nonnegative entries, unit row sums) for a stochastic matrix's p-th root to itself be stochastic — the algebraic condition behind Takada et al.'s [ID 350, Takada et al. 2010] yearly-root existence result.</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
@@ -16960,7 +17064,7 @@
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (abstract, §1).</t>
+          <t>Charitos, de Waal &amp; van der Gaag 2008 solves the same short-interval transition-matrix problem as Kingman [ID 382, Kingman 1962] and Israel et al. [ID 383, Israel et al. 2001] by regularisation, replacing invalid rows using a distance criterion rather than an algebraic fix.</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -17003,7 +17107,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Singer &amp; Spilerman 1976 surveys Markov-model representations of social processes, filed alongside the embedding-problem cluster [ID 382-385] as an applied precedent for discrete-time-interval Markov fitting; header-verified via a Columbia Academic Commons copy, unread.</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -17046,7 +17150,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§§3–4, Appendix C).</t>
+          <t>Reynolds &amp; Stoumbos 2000 develops an exact Markov-chain expression for the Bernoulli CUSUM chart's average run length (their Appendix C), turning framework row 2's Monte Carlo threshold into a check on an exact computation rather than the computation itself.</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -17089,7 +17193,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§§1–2, Table 1).</t>
+          <t>Lucas &amp; Crosier 1982 gives the fast-initial-response head start and Markov-chain average-run-length tables for the CUSUM chart, the companion tool to Reynolds &amp; Stoumbos's [ID 387, Reynolds &amp; Stoumbos 2000] exact ANOS expression for framework §17.7.</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -17132,7 +17236,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§2, Theorem 2.1).</t>
+          <t>Kaiser, Lahiri &amp; Nordman 2012 gives a goodness-of-fit test for exactly the autologistic model framework §15.1 fits, via generalized spatial residuals partitioned into concliques of mutually non-neighbouring sites (their Theorem 2.1) — a published diagnostic, not merely a fitting method.</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -17175,7 +17279,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read (§1).</t>
+          <t>Nordman &amp; Lahiri 2004 shows a subsample size proportional to n^(1/3) minimises the mean-squared error of a spatial variance estimate — a rule distinct from, and answering a different question than, Valavi et al.'s [ID 303, Valavi et al. 2018] block-size leakage rule for cross-validation.</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -17218,7 +17322,7 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read abstract.</t>
+          <t>Lahiri &amp; Zhu 2006 extends spatial resampling to irregular sampling designs, read at the abstract only, filed alongside Nordman &amp; Lahiri's [ID 390, Nordman &amp; Lahiri 2004] subsample-size rule for framework §13's variance-estimation cluster.</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -17261,7 +17365,7 @@
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read abstract (author working-paper copy).</t>
+          <t>Kelejian &amp; Prucha 2007 gives HAC standard-error estimation under spatial dependence — a correction for confidence intervals on a fitted score rather than an estimator for the score itself, read at the abstract only.</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -17304,7 +17408,7 @@
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Conley &amp; Molinari 2007 extends spatial-HAC standard errors to the case where location or distance itself carries measurement error — filed alongside Kelejian &amp; Prucha 2007 [ID 392, Kelejian &amp; Prucha 2007] for the same inference-correction role; a cemmap working paper, unread.</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -17347,7 +17451,7 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Politis &amp; Romano 1994 gives large-sample confidence regions from subsamples under minimal assumptions — the general subsampling theory behind Nordman &amp; Lahiri's [ID 390, Nordman &amp; Lahiri 2004] block-size rule; obtained only as an image-only scan, unread.</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -17390,7 +17494,7 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read abstract only (full PDF held).</t>
+          <t>Liu, Song, Townshend &amp; Gong 2008 multiplies a pixel-wise local probability of change by a global transition model in a space-time MRF for forest change detection — the multiplicative transition form (Hughes, Guttorp &amp; Charles 1999 [ID 314, Hughes et al. 1999]) already applied in remote sensing; read at the abstract only.</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
@@ -17433,7 +17537,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade filed-unread, no further reviewer note recorded in the bibliography.</t>
+          <t>Solberg, Taxt &amp; Jain 1996 is an early Markov random field classifier for multisource satellite imagery, filed alongside the applied space-time MRF cluster [ID 395, 404, 405] for framework §14.9's multiplicative transition precedent; header-verified, unread.</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -17476,7 +17580,7 @@
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Reynolds &amp; Stoumbos 1999 (*J. Quality Technology*, PRIMARY, §§2–3, Appendix A). "The properties of the Bernoulli CUSUM chart are evaluated using exact Markov chain methods". The construction: with `r₁ = −log((1−p₁)/(1−p₀))` and `r₂ = log(p₁(1−p₀)/ (p₀(1−p₁)))` (their Eq. 3, transcribed), choose `p₁` so that `r₂/r₁ = m` is an integer; the chart statistic then lives on multiples of `1/m`, state `i` is the value `(i−1)/m`, there are `t = m·h_B` transient states, and "after each observation the transition will either" go down one state or up `m − 1` states. The ANOS follows from the transient matrix (Appendix B).</t>
+          <t>Reynolds &amp; Stoumbos 1999 (J. Quality Technology, PRIMARY, §§2–3, Appendix A) states that Bernoulli CUSUM chart properties "are evaluated using exact Markov chain methods". The construction: with r₁ and r₂ as log-likelihood-ratio constants (their Eq. 3), choose p₁ so r₂/r₁ = m is an integer; the chart statistic then lives on multiples of 1/m across t = m·h_B transient states, moving down one state or up m−1 states per observation. The ANOS follows from the transient matrix (Appendix B).</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -17519,7 +17623,7 @@
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t>Zhu, Zheng, Carroll &amp; Aukema 2008 (*JABES*, PRIMARY, §§1–3). The paper that turns the 2005 model into ours: "we will modify the STARM so that the conditional distributions depend only on the past" — their Eq. 2.1, "the conditional distribution of Y t given the past depends on the most recent S time points" — a forward Markov chain in time with a Markov random field in space, i.e. framework §2 plus §3 exactly. On estimation: pseudo-likelihood.</t>
+          <t>Zhu, Zheng, Carroll &amp; Aukema 2008 (*JABES*, PRIMARY, §§1–3). The paper that turns the 2005 model into the one framework §2/§3 uses: "we will modify the STARM so that the conditional distributions depend only on the past" — their Eq. 2.1, "the conditional distribution of Y t given the past depends on the most recent S time points" — a forward Markov chain in time with a Markov random field in space, i.e. framework §2 plus §3 exactly. On estimation: pseudo-likelihood.</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
@@ -17605,7 +17709,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>Zhu, Zheng, Carroll &amp; Aukema 2008 (*JABES*, PRIMARY, §§1–3). The paper that turns the 2005 model into ours: "we will modify the STARM so that the conditional distributions depend only on the past" — their Eq. 2.1, "the conditional distribution of Y t given the past depends on the most recent S time points" — a forward Markov chain in time with a Markov random field in space, i.e. framework §2 plus §3 exactly. On estimation: pseudo-likelihood.</t>
+          <t>Zheng &amp; Zhu 2008 is the companion to Zhu, Zheng, Carroll &amp; Aukema 2008 (Zhu et al. 2008) [ID 398]: it proposes fitting the same spatial-temporal autologistic model by Markov chain Monte Carlo rather than the pseudo-likelihood estimator used there, an alternative estimation route for framework §2/§3's chain-plus-field structure. ABSTRACT grade — the reviewer has read the abstract only; the full PDF is held but not yet reviewed.</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -17777,7 +17881,7 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list. reviewer-read abstract (full PDF held).</t>
+          <t>Liu &amp; Cai 2012 reconstructs land-cover change trajectories from multi-temporal imagery by MRF trajectory modelling — an applied precedent for framework §14.9 alongside Cai et al. 2014 [ID 405, Cai et al. 2014] and Melgani &amp; Serpico 2003 [ID 406, Melgani &amp; Serpico 2003]; read at the abstract only.</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -17820,7 +17924,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>Filed under Round 9 (2026-09-12; §4.18) — seven fields named from the [D] list; grade ABSTRACT, no further reviewer note recorded in the bibliography.</t>
+          <t>Cai, Liu, Sulla-Menashe &amp; Friedl 2014 repairs illogical transitions in the MODIS land-cover product by a spatial-temporal modelling algorithm — the operational MRF-repair precedent alongside Liu &amp; Cai 2012 [ID 404, Liu &amp; Cai 2012]; read at the abstract only.</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -17949,7 +18053,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Jackson 2011 (*J. Statistical Software*, CC BY, PRIMARY, §§1.4, 2). The likelihood is the product over units and observation pairs of transition-matrix entries: "Each component Li,j is the entry of the transition matrix P(t) at the S(tij)th row and S(ti,j+1)th column, evaluated at t = ti,j+1 − tij". The hidden-Markov extension adds a misclassification matrix "where ers is the probability of observing state s conditionally on occupying true state r", and "The misclassification probabilities may also be modelled in terms of covariates" — which is exactly a band- and epoch-indexed emission. Fitted by `optim` on `log q_rs`, standard errors from the Hessian; software `msm`.</t>
+          <t>Jackson 2011 (J. Statistical Software, CC BY, PRIMARY, §§1.4, 2) gives the likelihood as the product over units and observation pairs of transition-matrix entries, each the P(t) entry at the row for the starting state and column for the ending state, evaluated at the interval between observations. The hidden-Markov extension adds a misclassification matrix where each entry is the probability of observing one state conditional on occupying another, with misclassification probabilities that may also depend on covariates — exactly a band- and epoch-indexed emission. Fitted by `optim` on `log q_rs` with standard errors from the Hessian; software `msm`.</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -18121,7 +18225,7 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Satten &amp; Longini 1996 (*Applied Statistics*, filed, header-verified, unread). van den Hout 2017 (book) not obtained.</t>
+          <t>Satten &amp; Longini 1996 model a Markov chain observed through measurement error to estimate the true course of an HIV marker; it is the earliest of the misclassified-state chain papers behind framework gap row 18 (transition rates attenuated by misclassification), alongside Rosychuk &amp; Thompson 2003 [ID 411, Rosychuk &amp; Thompson 2003]. Not yet read.</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -18164,7 +18268,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Gasparrini, Armstrong &amp; Kenward 2010 (*Statist. Med.*, author copy, PRIMARY, §3). The lag dimension is a vector of lagged exposures; a basis matrix `C` over lags turns it into `v` transformed covariates `W = Q·C` (their Eqs. 4–5), the implied lag effects are `b̂ = C ĝ` with covariance `C V(ĝ) Cᵀ` (Eq. 6), and "the choice of the basis to derive C can be considered as the application of a constraint to the shape of the distributed lag curve". A step-function basis is the histogram kernel of §4.18.4; a spline basis is a smooth one; the *cross-basis* extends it to a lag × dose (for us lag × distance) surface.</t>
+          <t>Gasparrini, Armstrong &amp; Kenward 2010 (Statist. Med., author copy, PRIMARY, §3) treats the lag dimension as a vector of lagged exposures: a basis matrix C over lags turns it into v transformed covariates `W = Q·C` (their Eqs. 4–5), with implied lag effects `b̂ = Cĝ` and covariance `C V(ĝ) Cᵀ` (Eq. 6). The choice of basis is itself a constraint on the shape of the distributed lag curve — a step-function basis is the histogram kernel of framework §4.18.4, a spline basis is a smooth one. The cross-basis extends it to a lag-by-dose (for the framework, lag-by-distance) surface.</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -18207,7 +18311,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Gasparrini 2011 (`dlnm`, ABSTRACT).</t>
+          <t>Gasparrini 2011 (`dlnm`) is the R package implementing the distributed-lag non-linear model's lag-basis construction (Gasparrini, Armstrong &amp; Kenward 2010 [ID 413, Gasparrini et al. 2010]) -- framework §19.2's lag-basis implementation; read at the abstract only.</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -18250,7 +18354,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read abstract.</t>
+          <t>Gasparrini 2014 extends the distributed-lag non-linear model to exposure-lag-response associations, generalising the lag-basis construction Gasparrini, Armstrong &amp; Kenward 2010 [ID 413, Gasparrini et al. 2010] and the `dlnm` package [ID 414, Gasparrini 2011] implement (framework §19.2); read at the abstract only.</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -18293,7 +18397,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read abstract.</t>
+          <t>Gasparrini, Scheipl, Armstrong &amp; Kenward 2017 fits the distributed-lag non-linear model with penalised splines inside a GAM, adding built-in model selection to the lag-basis construction of Gasparrini et al. 2010 [ID 413, Gasparrini et al. 2010]; read at the abstract only.</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -18336,7 +18440,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Almon 1965 (*Econometrica*, filed, header-verified, unread — the origin).</t>
+          <t>Almon 1965 is the origin of the distributed lag model (a polynomial lag basis in a regression), the lineage that Gasparrini, Armstrong &amp; Kenward 2010 [ID 413, Gasparrini et al. 2010] extend to the cross-basis used for framework gap row 19. Not yet read.</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -18422,7 +18526,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read opening.</t>
+          <t>Pillow et al. 2008 fits stimulus, post-spike and coupling filters as exponentiated linear terms in a point-process GLM — an applied instance of the self-exciting-kernel-as-regression form Truccolo et al. 2005 [ID 418, Truccolo et al. 2005] states in general, for framework §19.2's kernel; read at the opening only.</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -18508,7 +18612,7 @@
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>Lu &amp; Reynolds 2001 (*J. Quality Technology*, PRIMARY, abstract): for an AR(1) plus noise process, "CUSUM charts based on the original observations perform as well as CUSUM charts of residuals, except in the case in which the level of autocorrelation is high and the shift in the process mean is large", and a design method for the observations chart under autocorrelation is given. So the residual chart is not automatically the answer; the correlogram measurement decides which regime we are in.</t>
+          <t>Lu &amp; Reynolds 2001 (*J. Quality Technology*, PRIMARY, abstract): for an AR(1) plus noise process, "CUSUM charts based on the original observations perform as well as CUSUM charts of residuals, except in the case in which the level of autocorrelation is high and the shift in the process mean is large", and a design method for the observations chart under autocorrelation is given. So the residual chart is not automatically the answer; the correlogram measurement decides which regime applies.</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
@@ -18766,7 +18870,7 @@
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t>Steiner, Cook, Farewell &amp; Treasure 2000 (*Biostatistics*, PRIMARY, §2; browser fetch): the risk-adjusted CUSUM — "The risk adjustment is made though a likelihood score" per subject, i.e. per-unit increments from each unit's own pre-change probability. That is our band- and epoch-indexed increment `ℓ_{t,b}` under its published name.</t>
+          <t>Steiner, Cook, Farewell &amp; Treasure 2000 (*Biostatistics*, PRIMARY, §2; browser fetch): the risk-adjusted CUSUM — "The risk adjustment is made though a likelihood score" per subject, i.e. per-unit increments from each unit's own pre-change probability. That is the framework's band- and epoch-indexed increment `ℓ_{t,b}` under its published name.</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
@@ -18948,7 +19052,7 @@
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t>N/A — AISTATS 2015 / PMLR 38</t>
+          <t>arXiv:1407.7644</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
@@ -19024,7 +19128,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read abstract.</t>
+          <t>Raykar et al. 2010 estimates each labeller's error rates jointly with the latent true label by EM in a crowd-labelling setting — the multi-annotator route to framework §19.4's row-16 emission-identifiability problem, alongside Dawid &amp; Skene's [ID 435, Dawid &amp; Skene 1979] earlier EM origin; read at the abstract only.</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -19067,7 +19171,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read abstract.</t>
+          <t>Ratner et al. 2017 (Snorkel) combines multiple noisy labelling functions by a generative model that estimates each function's accuracy without ground truth — the weak-supervision route to framework §19.4's emission-identifiability problem, alongside Platanios et al.'s [ID 429, Platanios et al. 2014] three-classifier route; read at the abstract only.</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -19196,7 +19300,7 @@
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t>Mousavi &amp; Reynolds 2009 (*J. Quality Technology*, PRIMARY, abstract and §1) is the exact case: a proportion monitored from "binary observations that follow a two-state Markov chain model with first-order dependence". Their finding overturns §4.19.3's compromise: the Shewhart p-chart and the Bernoulli CUSUM "are not robust to autocorrelation, and that adjusting the control limits of these traditional charts to account for the autocorrelation is not an efficient approach". Instead they "construct a Markov binary CUSUM (MBCUSUM) chart based on a log-likelihood-ratio statistic" whose properties are again exact by a Markov chain. The increment of that chart is the log-likelihood ratio *under the dependent model* —.</t>
+          <t>Mousavi &amp; Reynolds 2009 (J. Quality Technology, PRIMARY, abstract and §1) is the exact case: a proportion monitored from binary observations following a two-state Markov chain with first-order dependence. Their finding overturns framework §4.19.3's compromise — the Shewhart p-chart and Bernoulli CUSUM "are not robust to autocorrelation", so they construct a Markov binary CUSUM (MBCUSUM) chart on a log-likelihood-ratio statistic whose properties are again exact by Markov chain. That increment is the chain's own evidence increment under the dependent model — framework row 20's dependence half is answered by a published chart, not by residuals or an adjusted limit.</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
@@ -19239,7 +19343,7 @@
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t>Hui &amp; Walter 1980 (*Biometrics*, PRIMARY, summary): two tests with unknown error rates applied to two populations with different prevalences, under conditional independence of the tests' errors, identify both tests' error rates and both prevalences — the two-population route to row 16's identifiability, complementary to Platanios's three-classifier route. For us: two strata with different canopy prevalence (e.g. two distance bands) and two arms.</t>
+          <t>Hui &amp; Walter 1980 (*Biometrics*, PRIMARY, summary): two tests with unknown error rates applied to two populations with different prevalences, under conditional independence of the tests' errors, identify both tests' error rates and both prevalences — the two-population route to framework gap row 16's identifiability, complementary to Platanios's three-classifier route. For the framework: two strata with different canopy prevalence (e.g. two distance bands) and two arms.</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
@@ -19325,7 +19429,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps. reviewer-read title/abstract (browser fetch).</t>
+          <t>Montgomery &amp; Mastrangelo 1991 surveys control-chart methods for autocorrelated data, part of the row-20 autocorrelated-CUSUM literature Lu &amp; Reynolds 2001 [ID 421, Lu &amp; Reynolds 2001] and Mousavi &amp; Reynolds 2009 [ID 437, Mousavi &amp; Reynolds 2009] build on; read at the title/abstract only via browser fetch.</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -19393,7 +19497,7 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Schwartz</t>
+          <t>Schwartz, J.</t>
         </is>
       </c>
       <c r="C443" t="n">
@@ -19401,10 +19505,14 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>[title not captured — see source note]</t>
-        </is>
-      </c>
-      <c r="E443" t="inlineStr"/>
+          <t>The Distributed Lag between Air Pollution and Daily Deaths</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Epidemiology</t>
+        </is>
+      </c>
       <c r="F443" t="inlineStr">
         <is>
           <t>Schwartz 2000 not obtained: absent from both Sci-Hub indexes; the agent stopped at two failed routes as instructed. Not load-bearing (Almon 1965 is the origin on file).</t>
@@ -19450,7 +19558,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>Filed under Round 10 (2026-09-12; §4.19) — the second-order gaps; grade METADATA, no further reviewer note recorded in the bibliography.</t>
+          <t>van den Hout's 2017 text extends multi-state survival modelling to interval-censored data, the book-length treatment of the irregular-interval panel-data problem Kalbfleisch &amp; Lawless 1985 [ID 407, Kalbfleisch &amp; Lawless 1985] and Jackson 2011 [ID 408, Jackson 2011] address in article form (framework §19.1); not obtained.</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
@@ -19493,7 +19601,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF). (local PDF; record and OA figures independently re-verified in round 2).</t>
+          <t>Li et al. 2026 (ALCC) produces temporally consistent annual land-cover maps over China 1985-2022 by an ensemble change-detection method — an operational-products precedent for framework §5's change-stratified reporting template (§4.11), read directly from a local PDF with its OA figures independently re-verified in round 2.</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -19536,7 +19644,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF); grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Artikanur et al. 2026 evaluates the accuracy and temporal consistency of several machine-learning LULC models in the Cimanuk watershed — a direct comparator for reporting per-year accuracy and temporal consistency together (framework §5); read directly from a local PDF.</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -19579,7 +19687,7 @@
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF). (already cited by `DEGRADED_IMAGERY_RESEARCH_2026-08-27.md`).</t>
+          <t>Van den Broeck, Goedeme &amp; Loopmans 2022 maps multiclass land cover from historical orthophotos using domain adaptation and spatio-temporal transfer learning — already cited by `DEGRADED_IMAGERY_RESEARCH_2026-08-27.md` for the cross-era imagery problem this project shares; read directly from a local PDF.</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
@@ -19622,7 +19730,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF); grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Maclaurin &amp; Leyk 2016 replicates the National Land Cover Database's classification temporally using active machine learning — a precedent for propagating one year's labels forward with model-in-the-loop correction, the same shape as this project's 2020-to-other-years projection; read directly from a local PDF.</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
@@ -19665,7 +19773,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF); grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Torres et al. 2021 detects deforestation with fully convolutional networks fused across Landsat-8 and Sentinel-2 in the Amazon — a multi-sensor change-detection precedent distinct from the single-sensor LandTrendr/CCDC family (framework §6.1); read directly from a local PDF.</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
@@ -19708,7 +19816,7 @@
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>Filed under the held-locally set (read directly from PDF); grade PRIMARY, no further reviewer note recorded in the bibliography.</t>
+          <t>Pearse, Watt, Soewarto &amp; Tan 2021 combines deep learning with phenological timing to classify tree species in aerial imagery during a biosecurity response — evidence that species-level phenology, not only sensor and season, drives per-epoch label disagreement (framework §1); read directly from a local PDF.</t>
         </is>
       </c>
       <c r="G450" t="inlineStr">
@@ -19751,7 +19859,7 @@
       </c>
       <c r="F451" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Boykov &amp; Kolmogorov 2003 formulates geodesics and minimal surfaces as graph cuts — filed unread among the round-9 graph-cut/max-flow search for a closed-form flip-threshold precedent behind the framework's [D] shrinking-bias claim (none found; Kolmogorov &amp; Boykov 2005 [ID 308, Kolmogorov &amp; Boykov 2005] states the verdict).</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
@@ -19794,7 +19902,7 @@
       </c>
       <c r="F452" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Vicente, Kolmogorov &amp; Rother 2008 adds connectivity priors to graph-cut segmentation and names the 'shrinking bias' explicitly in its abstract — filed unread among the same round-9 search for a closed-form flip threshold (none found beyond Kolmogorov &amp; Boykov 2005's [ID 308, Kolmogorov &amp; Boykov 2005] verdict).</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
@@ -19837,7 +19945,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Boykov &amp; Jolly 2001 is the interactive graph-cut segmentation paper the later shrinking-bias literature builds on — filed unread among the round-9 search for a closed-form flip threshold (none found beyond Kolmogorov &amp; Boykov 2005's [ID 308, Kolmogorov &amp; Boykov 2005] verdict).</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
@@ -19880,7 +19988,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Kolmogorov &amp; Zabih 2004 characterises which energy functions graph cuts can minimise exactly — filed unread among the round-9 search for a closed-form flip threshold behind the framework's [D] shrinking-bias claim (none found beyond Kolmogorov &amp; Boykov 2005's [ID 308, Kolmogorov &amp; Boykov 2005] verdict).</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
@@ -19923,7 +20031,7 @@
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Sinop &amp; Grady 2007 unifies graph cuts and the random-walker algorithm under one seeded-segmentation framework — filed unread among the round-9 search for a closed-form flip threshold (none found beyond Kolmogorov &amp; Boykov 2005's [ID 308, Kolmogorov &amp; Boykov 2005] verdict).</t>
         </is>
       </c>
       <c r="G455" t="inlineStr">
@@ -19966,7 +20074,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>Filed and searcher-verified but unread; one of the round-9 graph-cut / max-flow energy-minimisation citations searched for a closed-form flip-threshold precedent for the framework's [D] claim (none found; see Kolmogorov &amp; Boykov 2005's verdict, id 123).</t>
+          <t>Couprie, Grady, Najman &amp; Talbot 2011 (Power Watershed) unifies several graph-based segmentation optimisation frameworks including graph cuts — filed unread among the round-9 search for a closed-form flip threshold (none found beyond Kolmogorov &amp; Boykov 2005's [ID 308, Kolmogorov &amp; Boykov 2005] verdict).</t>
         </is>
       </c>
       <c r="G456" t="inlineStr">
@@ -20009,7 +20117,7 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>Obtained 2026-09-12 in the acquisition pass, header-verified, unread by the reviewer, as part of the round-9 search for the geometric-covariogram / erasure-radius literature behind framework §4.18; grade unchanged until read.</t>
+          <t>Blakemore 1984 addresses generalisation and error in spatial databases — sought in round 9 for the geometric-covariogram/erasure-radius literature behind framework §4.18; obtained in the acquisition pass, header-verified, unread.</t>
         </is>
       </c>
       <c r="G457" t="inlineStr">
@@ -20052,7 +20160,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Obtained 2026-09-12 in the acquisition pass, header-verified, unread by the reviewer, as part of the round-9 search for the geometric-covariogram / erasure-radius literature behind framework §4.18; grade unchanged until read.</t>
+          <t>Hall 1985 treats resampling of a coverage pattern in stochastic-process terms — sought in round 9 alongside Blakemore 1984 [ID 456, Blakemore 1984] for the same covariogram/erasure-radius literature (framework §4.18); obtained in the acquisition pass, header-verified, unread.</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
@@ -20077,7 +20185,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>Page</t>
+          <t>Page, E.S.</t>
         </is>
       </c>
       <c r="C459" t="n">
@@ -20085,7 +20193,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>[title not captured — still not obtained per the round-9 note]</t>
+          <t>Continuous Inspection Schemes</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
@@ -20095,7 +20203,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>Named in the round-9 geometric-covariogram / erasure-radius search (framework §4.18) but still not obtained — not in either Sci-Hub index checked.</t>
+          <t>Page 1954 is named in framework §4.18.6 as the origin of the CUSUM run-length problem that Reynolds &amp; Stoumbos 1999 (Reynolds &amp; Stoumbos 1999) [ID 397] and Lucas &amp; Crosier 1982 (Lucas &amp; Crosier 1982) [ID 388] build on. Still not obtained; not on the first Sci-Hub index checked.</t>
         </is>
       </c>
       <c r="G459" t="inlineStr">
@@ -20120,7 +20228,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>Lahiri</t>
+          <t>Lahiri, S.N.</t>
         </is>
       </c>
       <c r="C460" t="n">
@@ -20128,7 +20236,7 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>[title not captured — still not obtained per the round-9 note]</t>
+          <t>Resampling Methods for Spatial Data</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
@@ -20138,7 +20246,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>Named in the round-9 geometric-covariogram / erasure-radius search (framework §4.18) but still not obtained — not in either Sci-Hub index checked.</t>
+          <t>Lahiri 2003 is named in framework §4.18.8 (resampling for dependent data) as an unobtained companion to the block-size rule in Nordman &amp; Lahiri 2004 (Nordman &amp; Lahiri 2004) [ID 390]; the chapter's landing page carried no file. Still not obtained, alongside Hall 1985 (Hall 1985) [ID 457].</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -20154,6 +20262,49 @@
       <c r="I460" t="inlineStr">
         <is>
           <t>Not Obtained</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>460</v>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Locke, D.H., Ossola, A., Schmit, J.P. &amp; Grove, J.M.</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Sub-parcel scale analysis is needed to capture socially-driven canopy cover change in Baltimore, MD</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Landscape and Urban Planning</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Locke, Ossola, Schmit &amp; Grove 2025 is cited alongside Ock et al. 2024 [ID 326, Ock et al. 2024] and Steenberg, Robinson &amp; Duinker 2018 [ID 360, Steenberg et al. 2018] in framework §4.2 development-as-prior cluster: a sub-parcel-scale analysis is needed to capture socially-driven canopy cover change in Baltimore, arguing for finer spatial resolution than parcel-level redevelopment records provide. Closed and absent from the archive; METADATA grade, not obtained.</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>Spatiotemporal consistency review: acquisition pass</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.landurbplan.2024.105187</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>To Read</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: final consistency — review § tokens may carry sub-levels (convention updated), two obtained-unread rows lose their read grade; CSV twins regenerated; zero rule violations
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -20200,11 +20200,6 @@
           <t>To Read</t>
         </is>
       </c>
-      <c r="J359" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
-        </is>
-      </c>
       <c r="K359" t="inlineStr">
         <is>
           <t>framework §14.6</t>
@@ -20220,7 +20215,7 @@
       </c>
       <c r="P359" t="inlineStr">
         <is>
-          <t>read_status=obtained-unread -&gt; Status To Read (2026-09-13)</t>
+          <t>read_status=obtained-unread -&gt; Status To Read (2026-09-13); grade blanked 2026-09-13: obtained-unread carries no read grade</t>
         </is>
       </c>
     </row>
@@ -26587,11 +26582,6 @@
           <t>To Read</t>
         </is>
       </c>
-      <c r="J461" t="inlineStr">
-        <is>
-          <t>PRIMARY</t>
-        </is>
-      </c>
       <c r="K461" t="inlineStr">
         <is>
           <t>review §4.2</t>
@@ -26607,7 +26597,7 @@
       </c>
       <c r="P461" t="inlineStr">
         <is>
-          <t>bib read_status: obtained-unread | bib line 157 read_status=obtained-unread, txt_on_disk=yes -&gt; obtained but explicitly not yet read; kept To Read (already correct), grade kept PRIMARY since full text is on disk (2026-09-13).</t>
+          <t>bib read_status: obtained-unread | bib line 157 read_status=obtained-unread, txt_on_disk=yes -&gt; obtained but explicitly not yet read; kept To Read (already correct), grade kept PRIMARY since full text is on disk (2026-09-13).; grade blanked 2026-09-13: obtained-unread carries no read grade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Anna's Archive member route: first batches — 8 works obtained and header-verified (Wehmann 2015, Hoberg 2015, Wu 2017, Song 2026, Brown 2022, Cardille 2016, Hecht 2015, Yang 2021), tracker/bibliography/CSV twins updated; ten wrong-paper downloads caught by content verification and quarantined
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -11385,7 +11385,7 @@
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -11396,10 +11396,20 @@
       <c r="K216" t="inlineStr">
         <is>
           <t>framework §2.3</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Wehmann_2015_spatial-temporal-contextual-markovian-kernel</t>
         </is>
       </c>
       <c r="N216" t="n">
         <v>8</v>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>obtained 2026-09-13 via Anna's Archive member route</t>
+        </is>
       </c>
     </row>
     <row r="217">
@@ -11705,7 +11715,7 @@
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -11716,6 +11726,11 @@
       <c r="K221" t="inlineStr">
         <is>
           <t>review §4.1</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>Hoberg_2015_conditional-random-fields-multitemporal-multiscale</t>
         </is>
       </c>
       <c r="N221" t="n">
@@ -11723,7 +11738,7 @@
       </c>
       <c r="P221" t="inlineStr">
         <is>
-          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Hoberg et al. 2015"</t>
+          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Hoberg et al. 2015" | obtained 2026-09-13 via Anna's Archive member route</t>
         </is>
       </c>
     </row>
@@ -12529,7 +12544,7 @@
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J235" t="inlineStr">
@@ -12540,10 +12555,20 @@
       <c r="K235" t="inlineStr">
         <is>
           <t>review §4.2</t>
+        </is>
+      </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Cardille_2016_bayesian-updating-land-cover</t>
         </is>
       </c>
       <c r="N235" t="n">
         <v>29</v>
+      </c>
+      <c r="P235" t="inlineStr">
+        <is>
+          <t>obtained 2026-09-13 via Anna's Archive member route</t>
+        </is>
       </c>
     </row>
     <row r="236">
@@ -13254,12 +13279,17 @@
           <t>ABSTRACT</t>
         </is>
       </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Song_2026_monocular-height-sparse-lidar-correction</t>
+        </is>
+      </c>
       <c r="N247" t="n">
         <v>46</v>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>lead restatement moved from Relevance: "Song et al. 2026"; Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read</t>
+          <t>lead restatement moved from Relevance: "Song et al. 2026"; Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read | obtained 2026-09-13 via open access (arXiv, curl) — Anna's Archive fetch was mis-matched to an unrelated paper and quarantined</t>
         </is>
       </c>
     </row>
@@ -13508,12 +13538,17 @@
           <t>review §4.4</t>
         </is>
       </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Brown_2022_aerial-animal-detection-spatial-resolution</t>
+        </is>
+      </c>
       <c r="N251" t="n">
         <v>50</v>
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>lead restatement moved from Relevance: "Brown et al. 2022"; Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read</t>
+          <t>lead restatement moved from Relevance: "Brown et al. 2022"; Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read | obtained 2026-09-13 via open access (arXiv, curl) — Anna's Archive fetch was mis-matched to an unrelated paper and quarantined</t>
         </is>
       </c>
     </row>
@@ -14738,12 +14773,17 @@
           <t>review §4.5</t>
         </is>
       </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>Wu_2017_iterative-slow-feature-change-detection</t>
+        </is>
+      </c>
       <c r="N271" t="n">
         <v>77</v>
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read</t>
+          <t>Status set Read 2026-09-13 by rule: grade ABSTRACT = abstract read | obtained 2026-09-13 via Anna's Archive member route</t>
         </is>
       </c>
     </row>
@@ -14842,7 +14882,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -14853,10 +14893,20 @@
       <c r="K273" t="inlineStr">
         <is>
           <t>framework §6.2; review §4.10</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>Hecht_2015_automatic-identification-building-types</t>
         </is>
       </c>
       <c r="N273" t="n">
         <v>79</v>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>obtained 2026-09-13 via Anna's Archive member route</t>
+        </is>
       </c>
     </row>
     <row r="274">
@@ -15254,16 +15304,26 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
         <is>
           <t>METADATA</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>Yang_2021_30m-annual-land-cover-china</t>
         </is>
       </c>
       <c r="N280" t="n">
         <v>86</v>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>obtained 2026-09-13 via open access (Copernicus, curl)</t>
+        </is>
       </c>
     </row>
     <row r="281">

</xml_diff>

<commit_message>
literature: Page 1954 obtained via its JSTOR DOI 10.2307/2333009 (Anna's Archive member route, verified), tracker row 458 and review bibliography updated
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -26517,7 +26517,7 @@
       </c>
       <c r="I459" t="inlineStr">
         <is>
-          <t>Not Obtained</t>
+          <t>To Read</t>
         </is>
       </c>
       <c r="J459" t="inlineStr">
@@ -26528,6 +26528,11 @@
       <c r="K459" t="inlineStr">
         <is>
           <t>review §4.18.6</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>Page_1954_continuous-inspection-schemes</t>
         </is>
       </c>
       <c r="N459" t="n">
@@ -26535,7 +26540,7 @@
       </c>
       <c r="P459" t="inlineStr">
         <is>
-          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Page 1954"</t>
+          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Page 1954" | obtained 2026-09-13 via annas-archive member API (verified gates; DOI 10.2307/2333009)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: Page 1954 row states its role in the CUSUM lineage (review §4.18.6, gap row 2) instead of acquisition status; DOI set to the JSTOR DOI used, OUP DOI kept in Notes; bibliography index row 246 notes the filing
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -26502,7 +26502,7 @@
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t>Is named in framework §4.18.6 as the origin of the CUSUM run-length problem that Reynolds &amp; Stoumbos 1999 [ID 397] and Lucas &amp; Crosier 1982 [ID 388] build on. Still not obtained; not on the first Sci-Hub index checked.</t>
+          <t>Cited in review §4.18.6 alongside Brook &amp; Evans 1972 [ID 402], Lucas &amp; Crosier 1982 [ID 388] and Reynolds &amp; Stoumbos 1999 [ID 397] as the origin of the CUSUM scheme behind framework gap row 2's Bernoulli-CUSUM detector (§17.7, §17.10 area). Cited only for that lineage; the paper itself is unread.</t>
         </is>
       </c>
       <c r="G459" t="inlineStr">
@@ -26512,7 +26512,7 @@
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1093/biomet/41.1-2.100</t>
+          <t>https://doi.org/10.2307/2333009</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
@@ -26540,7 +26540,7 @@
       </c>
       <c r="P459" t="inlineStr">
         <is>
-          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Page 1954" | obtained 2026-09-13 via annas-archive member API (verified gates; DOI 10.2307/2333009)</t>
+          <t>bib read_status: obtained-unread | lead restatement moved from Relevance: "Page 1954" | obtained 2026-09-13 via annas-archive member API (verified gates; DOI 10.2307/2333009) | also registered as 10.1093/biomet/41.1-2.100</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
literature: correct two DOIs that belonged to other papers (Averkov & Bianchi 2009 -> 10.4171/jems/179; Higham & Lin 2011 -> 10.1016/j.laa.2010.04.007), found by the fast audit and confirmed on Crossref; review bibliography, index, rename map, tracker rows 367/384 and CSV twin
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MUcyGTfX2koRdYAjW5kED
</commit_message>
<xml_diff>
--- a/Literature_Tracker.xlsx
+++ b/Literature_Tracker.xlsx
@@ -20826,7 +20826,7 @@
       </c>
       <c r="H368" t="inlineStr">
         <is>
-          <t>https://doi.org/10.4171/jems/183</t>
+          <t>https://doi.org/10.4171/jems/179</t>
         </is>
       </c>
       <c r="I368" t="inlineStr">
@@ -20849,7 +20849,7 @@
       </c>
       <c r="P368" t="inlineStr">
         <is>
-          <t>bib grade not yet resolved (filed-unread); bib read_status: obtained-unread</t>
+          <t>bib grade not yet resolved (filed-unread); bib read_status: obtained-unread; DOI corrected 2026-09-13 (was 10.4171/JEMS/183, which is a different paper)</t>
         </is>
       </c>
     </row>
@@ -21903,7 +21903,7 @@
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>https://doi.org/10.1016/j.laa.2010.09.001</t>
+          <t>https://doi.org/10.1016/j.laa.2010.04.007</t>
         </is>
       </c>
       <c r="I385" t="inlineStr">
@@ -21926,7 +21926,7 @@
       </c>
       <c r="P385" t="inlineStr">
         <is>
-          <t>bib read_status: reviewer-read</t>
+          <t>bib read_status: reviewer-read; DOI corrected 2026-09-13 (was 10.1016/j.laa.2010.09.001, which is a different paper)</t>
         </is>
       </c>
     </row>

</xml_diff>